<commit_message>
LC -> LU conversion: - Reorganized workflow and scenarios
</commit_message>
<xml_diff>
--- a/src/LULUCF/scripts/postprocessing/conversion_LUC_scenarios.xlsx
+++ b/src/LULUCF/scripts/postprocessing/conversion_LUC_scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\scripts\postprocessing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D711A765-EA99-40FA-B51B-0881170739A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47FE53F1-2657-48F1-87CE-4B36D5CA164A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="51">
   <si>
     <t>Driver</t>
   </si>
@@ -144,15 +144,6 @@
     <t>id</t>
   </si>
   <si>
-    <t>lc_2000</t>
-  </si>
-  <si>
-    <t>lc_2005</t>
-  </si>
-  <si>
-    <t>lc_2010</t>
-  </si>
-  <si>
     <t>lc_2015</t>
   </si>
   <si>
@@ -189,9 +180,6 @@
     <t>After tall vegetation is established, short veg is considered forest since SDPT</t>
   </si>
   <si>
-    <t>After tall vegetation is established, cultivated grassland is considered forest since SDPT</t>
-  </si>
-  <si>
     <t xml:space="preserve">Forest the entire time series because logging concession </t>
   </si>
   <si>
@@ -207,12 +195,6 @@
     <t>Forest remaining forest (if n_years_unstocked_forest = 5)</t>
   </si>
   <si>
-    <t>Forest to grassland (because it is cultivated grass)</t>
-  </si>
-  <si>
-    <t>Forest to grassland in interior interval, but not at the end because Logging driver</t>
-  </si>
-  <si>
     <t>Forest to cropland in 2022</t>
   </si>
   <si>
@@ -229,6 +211,9 @@
   </si>
   <si>
     <t>Back and foth between Forest and cropland until 2018?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* </t>
   </si>
 </sst>
 </file>
@@ -313,7 +298,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill>
@@ -325,34 +310,6 @@
       <fill>
         <patternFill>
           <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF8ABE66"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -655,17 +612,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="8"/>
-    <col min="15" max="15" width="9.21875" customWidth="1"/>
-    <col min="16" max="16" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.21875" customWidth="1"/>
+    <col min="13" max="13" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>26</v>
       </c>
@@ -699,43 +656,34 @@
       <c r="K1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="O1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="P1" t="s">
+      <c r="M1" t="s">
         <v>24</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="N1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -747,113 +695,89 @@
         <v>1</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
         <v>1</v>
       </c>
       <c r="N2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>3</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M3">
         <v>2</v>
       </c>
-      <c r="N3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>3</v>
       </c>
       <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
       <c r="D4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>3</v>
       </c>
       <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
         <v>3</v>
       </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
       <c r="H4">
         <v>1</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4">
         <v>3</v>
       </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-      <c r="N4">
-        <v>1</v>
-      </c>
-      <c r="O4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -861,51 +785,39 @@
         <v>3</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5">
         <v>3</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5">
         <v>3</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>3</v>
       </c>
       <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-      <c r="N5">
-        <v>2</v>
-      </c>
-      <c r="O5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -914,7 +826,7 @@
         <v>1</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6">
         <v>3</v>
@@ -932,69 +844,48 @@
         <v>3</v>
       </c>
       <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-      <c r="N6">
-        <v>1</v>
-      </c>
-      <c r="P6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L7">
-        <v>2</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
-      </c>
-      <c r="N7">
-        <v>2</v>
-      </c>
-      <c r="P7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -1005,13 +896,13 @@
         <v>3</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -1028,180 +919,139 @@
       <c r="K8">
         <v>1</v>
       </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8">
-        <v>1</v>
-      </c>
-      <c r="N8">
-        <v>1</v>
-      </c>
-      <c r="Q8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>8</v>
       </c>
-      <c r="B9">
-        <v>3</v>
-      </c>
-      <c r="C9">
-        <v>3</v>
-      </c>
-      <c r="D9">
-        <v>3</v>
-      </c>
-      <c r="E9">
-        <v>3</v>
-      </c>
-      <c r="F9">
-        <v>3</v>
-      </c>
-      <c r="G9">
-        <v>2</v>
-      </c>
-      <c r="H9">
-        <v>2</v>
-      </c>
-      <c r="I9">
-        <v>2</v>
-      </c>
-      <c r="J9">
-        <v>3</v>
-      </c>
-      <c r="K9">
-        <v>3</v>
-      </c>
-      <c r="L9">
-        <v>2</v>
-      </c>
-      <c r="M9">
-        <v>2</v>
-      </c>
-      <c r="N9">
-        <v>2</v>
-      </c>
-      <c r="Q9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B9" s="1">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1">
+        <v>7</v>
+      </c>
+      <c r="E9" s="1">
+        <v>7</v>
+      </c>
+      <c r="F9" s="1">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1">
+        <v>7</v>
+      </c>
+      <c r="H9" s="1">
+        <v>7</v>
+      </c>
+      <c r="I9" s="1">
+        <v>7</v>
+      </c>
+      <c r="J9" s="1">
+        <v>7</v>
+      </c>
+      <c r="K9" s="1">
+        <v>7</v>
+      </c>
+      <c r="L9" s="6"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>9</v>
       </c>
       <c r="B10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J10" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K10" s="1">
-        <v>7</v>
-      </c>
-      <c r="L10" s="1">
-        <v>7</v>
-      </c>
-      <c r="M10" s="1">
-        <v>7</v>
-      </c>
-      <c r="N10" s="1">
-        <v>7</v>
-      </c>
-      <c r="O10" s="6"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="L10" s="6"/>
+    </row>
+    <row r="11" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>10</v>
       </c>
       <c r="B11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J11" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K11" s="1">
-        <v>5</v>
-      </c>
-      <c r="L11" s="1">
-        <v>5</v>
-      </c>
-      <c r="M11" s="1">
-        <v>5</v>
-      </c>
-      <c r="N11" s="1">
-        <v>5</v>
-      </c>
-      <c r="O11" s="6"/>
-    </row>
-    <row r="12" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="L11" s="6"/>
+    </row>
+    <row r="12" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>11</v>
       </c>
       <c r="B12" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C12" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D12" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E12" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F12" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G12" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H12" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I12" s="1">
         <v>10</v>
@@ -1212,18 +1062,9 @@
       <c r="K12" s="1">
         <v>10</v>
       </c>
-      <c r="L12" s="1">
-        <v>10</v>
-      </c>
-      <c r="M12" s="1">
-        <v>10</v>
-      </c>
-      <c r="N12" s="1">
-        <v>10</v>
-      </c>
-      <c r="O12" s="6"/>
-    </row>
-    <row r="13" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="L12" s="7"/>
+    </row>
+    <row r="13" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>12</v>
       </c>
@@ -1249,26 +1090,19 @@
         <v>7</v>
       </c>
       <c r="I13" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J13" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K13" s="1">
-        <v>7</v>
-      </c>
-      <c r="L13" s="1">
-        <v>10</v>
-      </c>
-      <c r="M13" s="1">
-        <v>10</v>
-      </c>
-      <c r="N13" s="1">
-        <v>10</v>
-      </c>
-      <c r="O13" s="7"/>
-    </row>
-    <row r="14" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="L13" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>13</v>
       </c>
@@ -1279,10 +1113,10 @@
         <v>7</v>
       </c>
       <c r="D14" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E14" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F14" s="1">
         <v>7</v>
@@ -1294,28 +1128,19 @@
         <v>7</v>
       </c>
       <c r="I14" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J14" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K14" s="1">
-        <v>7</v>
-      </c>
-      <c r="L14" s="1">
-        <v>10</v>
-      </c>
-      <c r="M14" s="1">
-        <v>10</v>
-      </c>
-      <c r="N14" s="1">
-        <v>10</v>
-      </c>
-      <c r="O14" s="7">
+        <v>10</v>
+      </c>
+      <c r="L14" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>14</v>
       </c>
@@ -1329,54 +1154,45 @@
         <v>7</v>
       </c>
       <c r="E15" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F15" s="1">
         <v>7</v>
       </c>
       <c r="G15" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H15" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I15" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J15" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K15" s="1">
-        <v>7</v>
-      </c>
-      <c r="L15" s="1">
-        <v>10</v>
-      </c>
-      <c r="M15" s="1">
-        <v>10</v>
-      </c>
-      <c r="N15" s="1">
-        <v>10</v>
-      </c>
-      <c r="O15" s="7">
+        <v>10</v>
+      </c>
+      <c r="L15" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>15</v>
       </c>
       <c r="B16" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C16" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D16" s="1">
         <v>7</v>
       </c>
       <c r="E16" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F16" s="1">
         <v>7</v>
@@ -1385,78 +1201,58 @@
         <v>7</v>
       </c>
       <c r="H16" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I16" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J16" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K16" s="1">
-        <v>7</v>
-      </c>
-      <c r="L16" s="1">
-        <v>10</v>
-      </c>
-      <c r="M16" s="1">
-        <v>10</v>
-      </c>
-      <c r="N16" s="1">
-        <v>10</v>
-      </c>
-      <c r="O16" s="7">
+        <v>5</v>
+      </c>
+      <c r="L16" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>16</v>
       </c>
       <c r="B17" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C17" s="1">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D17" s="1">
         <v>7</v>
       </c>
       <c r="E17" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F17" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G17" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H17" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I17" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J17" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K17" s="1">
-        <v>7</v>
-      </c>
-      <c r="L17" s="1">
-        <v>5</v>
-      </c>
-      <c r="M17" s="1">
-        <v>5</v>
-      </c>
-      <c r="N17" s="1">
-        <v>5</v>
-      </c>
-      <c r="O17" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="L17" s="7"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>17</v>
       </c>
@@ -1464,13 +1260,13 @@
         <v>7</v>
       </c>
       <c r="C18" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D18" s="1">
         <v>7</v>
       </c>
       <c r="E18" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F18" s="1">
         <v>7</v>
@@ -1479,72 +1275,18 @@
         <v>7</v>
       </c>
       <c r="H18" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I18" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J18" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="K18" s="1">
-        <v>10</v>
-      </c>
-      <c r="L18" s="1">
-        <v>10</v>
-      </c>
-      <c r="M18" s="1">
-        <v>10</v>
-      </c>
-      <c r="N18" s="1">
-        <v>10</v>
-      </c>
-      <c r="O18" s="7"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A19" s="8">
-        <v>18</v>
-      </c>
-      <c r="B19" s="1">
-        <v>7</v>
-      </c>
-      <c r="C19" s="1">
-        <v>7</v>
-      </c>
-      <c r="D19" s="1">
-        <v>7</v>
-      </c>
-      <c r="E19" s="1">
-        <v>7</v>
-      </c>
-      <c r="F19" s="1">
-        <v>7</v>
-      </c>
-      <c r="G19" s="1">
-        <v>7</v>
-      </c>
-      <c r="H19" s="1">
-        <v>7</v>
-      </c>
-      <c r="I19" s="1">
-        <v>7</v>
-      </c>
-      <c r="J19" s="1">
-        <v>7</v>
-      </c>
-      <c r="K19" s="1">
-        <v>7</v>
-      </c>
-      <c r="L19" s="1">
-        <v>7</v>
-      </c>
-      <c r="M19" s="1">
-        <v>7</v>
-      </c>
-      <c r="N19" s="1">
-        <v>7</v>
-      </c>
-      <c r="O19" s="7">
+        <v>7</v>
+      </c>
+      <c r="L18" s="7">
         <v>3</v>
       </c>
     </row>
@@ -1555,15 +1297,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FD5E73A-BF21-4771-A2AF-1B9A394A8B1D}">
-  <dimension ref="A1:W69"/>
+  <dimension ref="A1:T65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="31.109375" customWidth="1"/>
+    <col min="12" max="12" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="31.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>2</v>
       </c>
@@ -1604,25 +1345,16 @@
         <v>14</v>
       </c>
       <c r="O1">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P1">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="Q1">
-        <v>17</v>
-      </c>
-      <c r="R1">
-        <v>18</v>
-      </c>
-      <c r="S1">
-        <v>19</v>
-      </c>
-      <c r="T1">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>26</v>
       </c>
@@ -1656,1501 +1388,1361 @@
       <c r="K2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q2" t="s">
         <v>37</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="P2" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>25</v>
-      </c>
-      <c r="T2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>1</v>
       </c>
       <c r="B3" t="str" cm="1">
-        <f t="array" ref="B3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="B3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="C3" t="str" cm="1">
-        <f t="array" ref="C3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D3" t="str" cm="1">
-        <f t="array" ref="D3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="E3" t="str" cm="1">
-        <f t="array" ref="E3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F3" t="str" cm="1">
-        <f t="array" ref="F3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="G3" t="str" cm="1">
-        <f t="array" ref="G3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H3" t="str" cm="1">
-        <f t="array" ref="H3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I3" t="str" cm="1">
-        <f t="array" ref="I3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J3" t="str" cm="1">
-        <f t="array" ref="J3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K3" t="str" cm="1">
-        <f t="array" ref="K3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L3" t="str" cm="1">
-        <f t="array" ref="L3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="L3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M3" t="str" cm="1">
-        <f t="array" ref="M3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="M3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N3" t="str" cm="1">
-        <f t="array" ref="N3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="O3" t="str" cm="1">
-        <f t="array" ref="O3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P3" t="str" cm="1">
-        <f t="array" ref="P3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q3" t="str" cm="1">
-        <f t="array" ref="Q3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v>yes</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>2</v>
       </c>
       <c r="B4" t="str" cm="1">
-        <f t="array" ref="B4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="B4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="C4" t="str" cm="1">
-        <f t="array" ref="C4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="C4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="D4" t="str" cm="1">
-        <f t="array" ref="D4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="E4" t="str" cm="1">
-        <f t="array" ref="E4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F4" t="str" cm="1">
-        <f t="array" ref="F4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="G4" t="str" cm="1">
-        <f t="array" ref="G4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="G4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="H4" t="str" cm="1">
-        <f t="array" ref="H4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="H4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="I4" t="str" cm="1">
-        <f t="array" ref="I4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="I4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="J4" t="str" cm="1">
-        <f t="array" ref="J4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K4" t="str" cm="1">
-        <f t="array" ref="K4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L4" t="str" cm="1">
-        <f t="array" ref="L4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="L4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M4" t="str" cm="1">
-        <f t="array" ref="M4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="M4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v>wood fiber</v>
       </c>
       <c r="N4" t="str" cm="1">
-        <f t="array" ref="N4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
-      </c>
-      <c r="O4" t="str" cm="1">
-        <f t="array" ref="O4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P4" t="str" cm="1">
-        <f t="array" ref="P4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q4" t="str" cm="1">
-        <f t="array" ref="Q4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>3</v>
       </c>
       <c r="B5" t="str" cm="1">
-        <f t="array" ref="B5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="B5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="C5" t="str" cm="1">
-        <f t="array" ref="C5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="C5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="D5" t="str" cm="1">
-        <f t="array" ref="D5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="E5" t="str" cm="1">
-        <f t="array" ref="E5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F5" t="str" cm="1">
-        <f t="array" ref="F5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="G5" t="str" cm="1">
-        <f t="array" ref="G5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="G5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="H5" t="str" cm="1">
-        <f t="array" ref="H5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I5" t="str" cm="1">
-        <f t="array" ref="I5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="I5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="J5" t="str" cm="1">
-        <f t="array" ref="J5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K5" t="str" cm="1">
-        <f t="array" ref="K5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="L5" t="str" cm="1">
-        <f t="array" ref="L5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="L5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M5" t="str" cm="1">
-        <f t="array" ref="M5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="M5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N5" t="str" cm="1">
-        <f t="array" ref="N5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="O5" t="str" cm="1">
-        <f t="array" ref="O5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Logging</v>
-      </c>
-      <c r="P5" t="str" cm="1">
-        <f t="array" ref="P5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q5" t="str" cm="1">
-        <f t="array" ref="Q5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>4</v>
       </c>
       <c r="B6" t="str" cm="1">
-        <f t="array" ref="B6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C6" t="str" cm="1">
-        <f t="array" ref="C6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="C6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="D6" t="str" cm="1">
-        <f t="array" ref="D6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E6" t="str" cm="1">
-        <f t="array" ref="E6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F6" t="str" cm="1">
-        <f t="array" ref="F6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G6" t="str" cm="1">
-        <f t="array" ref="G6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="G6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="H6" t="str" cm="1">
-        <f t="array" ref="H6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="H6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="I6" t="str" cm="1">
-        <f t="array" ref="I6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="I6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="J6" t="str" cm="1">
-        <f t="array" ref="J6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K6" t="str" cm="1">
-        <f t="array" ref="K6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L6" t="str" cm="1">
-        <f t="array" ref="L6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="L6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M6" t="str" cm="1">
-        <f t="array" ref="M6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="M6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N6" t="str" cm="1">
-        <f t="array" ref="N6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
-      </c>
-      <c r="O6" t="str" cm="1">
-        <f t="array" ref="O6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Logging</v>
-      </c>
-      <c r="P6" t="str" cm="1">
-        <f t="array" ref="P6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q6" t="str" cm="1">
-        <f t="array" ref="Q6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>5</v>
       </c>
       <c r="B7" t="str" cm="1">
-        <f t="array" ref="B7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="B7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="C7" t="str" cm="1">
-        <f t="array" ref="C7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D7" t="str" cm="1">
-        <f t="array" ref="D7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E7" t="str" cm="1">
-        <f t="array" ref="E7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F7" t="str" cm="1">
-        <f t="array" ref="F7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G7" t="str" cm="1">
-        <f t="array" ref="G7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H7" t="str" cm="1">
-        <f t="array" ref="H7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I7" t="str" cm="1">
-        <f t="array" ref="I7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J7" t="str" cm="1">
-        <f t="array" ref="J7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K7" t="str" cm="1">
-        <f t="array" ref="K7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L7" t="str" cm="1">
-        <f t="array" ref="L7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="L7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M7" t="str" cm="1">
-        <f t="array" ref="M7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="M7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N7" t="str" cm="1">
-        <f t="array" ref="N7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="O7" t="str" cm="1">
-        <f t="array" ref="O7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P7" t="str" cm="1">
-        <f t="array" ref="P7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v>wood fiber</v>
-      </c>
-      <c r="Q7" t="str" cm="1">
-        <f t="array" ref="Q7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>6</v>
       </c>
       <c r="B8" t="str" cm="1">
-        <f t="array" ref="B8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="B8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="C8" t="str" cm="1">
-        <f t="array" ref="C8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="C8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="D8" t="str" cm="1">
-        <f t="array" ref="D8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="D8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="E8" t="str" cm="1">
-        <f t="array" ref="E8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F8" t="str" cm="1">
-        <f t="array" ref="F8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="G8" t="str" cm="1">
-        <f t="array" ref="G8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="G8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="H8" t="str" cm="1">
-        <f t="array" ref="H8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="H8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="I8" t="str" cm="1">
-        <f t="array" ref="I8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="I8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="J8" t="str" cm="1">
-        <f t="array" ref="J8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K8" t="str" cm="1">
-        <f t="array" ref="K8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L8" t="str" cm="1">
-        <f t="array" ref="L8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="L8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Logging</v>
       </c>
       <c r="M8" t="str" cm="1">
-        <f t="array" ref="M8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="M8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N8" t="str" cm="1">
-        <f t="array" ref="N8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
-      </c>
-      <c r="O8" t="str" cm="1">
-        <f t="array" ref="O8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P8" t="str" cm="1">
-        <f t="array" ref="P8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v>wood fiber</v>
-      </c>
-      <c r="Q8" t="str" cm="1">
-        <f t="array" ref="Q8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T8" t="s">
+        <f t="array" ref="N8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A9" s="8">
+        <v>7</v>
+      </c>
+      <c r="B9" t="str" cm="1">
+        <f t="array" ref="B9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C9" t="str" cm="1">
+        <f t="array" ref="C9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D9" t="str" cm="1">
+        <f t="array" ref="D9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="E9" t="str" cm="1">
+        <f t="array" ref="E9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="F9" t="str" cm="1">
+        <f t="array" ref="F9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="G9" t="str" cm="1">
+        <f t="array" ref="G9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="H9" t="str" cm="1">
+        <f t="array" ref="H9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="I9" t="str" cm="1">
+        <f t="array" ref="I9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="J9" t="str" cm="1">
+        <f t="array" ref="J9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="K9" t="str" cm="1">
+        <f t="array" ref="K9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="L9" t="str" cm="1">
+        <f t="array" ref="L9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M9" t="str" cm="1">
+        <f t="array" ref="M9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="N9" t="str" cm="1">
+        <f t="array" ref="N9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A9" s="8">
-        <v>7</v>
-      </c>
-      <c r="B9" t="str" cm="1">
-        <f t="array" ref="B9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="C9" t="str" cm="1">
-        <f t="array" ref="C9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="D9" t="str" cm="1">
-        <f t="array" ref="D9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="E9" t="str" cm="1">
-        <f t="array" ref="E9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="F9" t="str" cm="1">
-        <f t="array" ref="F9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="G9" t="str" cm="1">
-        <f t="array" ref="G9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="H9" t="str" cm="1">
-        <f t="array" ref="H9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="I9" t="str" cm="1">
-        <f t="array" ref="I9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="J9" t="str" cm="1">
-        <f t="array" ref="J9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="K9" t="str" cm="1">
-        <f t="array" ref="K9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="L9" t="str" cm="1">
-        <f t="array" ref="L9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="M9" t="str" cm="1">
-        <f t="array" ref="M9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="N9" t="str" cm="1">
-        <f t="array" ref="N9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="O9" t="str" cm="1">
-        <f t="array" ref="O9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P9" t="str" cm="1">
-        <f t="array" ref="P9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q9" t="str" cm="1">
-        <f t="array" ref="Q9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v>yes</v>
-      </c>
-      <c r="T9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>8</v>
       </c>
       <c r="B10" t="str" cm="1">
-        <f t="array" ref="B10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C10" t="str" cm="1">
-        <f t="array" ref="C10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D10" t="str" cm="1">
-        <f t="array" ref="D10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E10" t="str" cm="1">
-        <f t="array" ref="E10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F10" t="str" cm="1">
-        <f t="array" ref="F10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G10" t="str" cm="1">
-        <f t="array" ref="G10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="G10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="H10" t="str" cm="1">
-        <f t="array" ref="H10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="H10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="I10" t="str" cm="1">
-        <f t="array" ref="I10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="I10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="J10" t="str" cm="1">
-        <f t="array" ref="J10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K10" t="str" cm="1">
-        <f t="array" ref="K10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="L10" t="str" cm="1">
-        <f t="array" ref="L10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="L10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M10" t="str" cm="1">
-        <f t="array" ref="M10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
+        <f t="array" ref="M10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N10" t="str" cm="1">
-        <f t="array" ref="N10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cultivated</v>
-      </c>
-      <c r="O10" t="str" cm="1">
-        <f t="array" ref="O10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P10" t="str" cm="1">
-        <f t="array" ref="P10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q10" t="str" cm="1">
-        <f t="array" ref="Q10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v>yes</v>
-      </c>
-      <c r="T10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>9</v>
       </c>
       <c r="B11" t="str" cm="1">
-        <f t="array" ref="B11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="B11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="C11" t="str" cm="1">
-        <f t="array" ref="C11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="C11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="D11" t="str" cm="1">
-        <f t="array" ref="D11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="E11" t="str" cm="1">
-        <f t="array" ref="E11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F11" t="str" cm="1">
-        <f t="array" ref="F11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="G11" t="str" cm="1">
-        <f t="array" ref="G11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="G11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="H11" t="str" cm="1">
-        <f t="array" ref="H11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="H11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="I11" t="str" cm="1">
-        <f t="array" ref="I11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="I11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="J11" t="str" cm="1">
-        <f t="array" ref="J11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K11" t="str" cm="1">
-        <f t="array" ref="K11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L11" t="str" cm="1">
-        <f t="array" ref="L11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="L11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M11" t="str" cm="1">
-        <f t="array" ref="M11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="M11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N11" t="str" cm="1">
-        <f t="array" ref="N11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="O11" t="str" cm="1">
-        <f t="array" ref="O11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P11" t="str" cm="1">
-        <f t="array" ref="P11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q11" t="str" cm="1">
-        <f t="array" ref="Q11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T11" t="s">
+        <f t="array" ref="N11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q11" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="T11" s="9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>10</v>
       </c>
       <c r="B12" t="str" cm="1">
-        <f t="array" ref="B12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="B12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="C12" t="str" cm="1">
-        <f t="array" ref="C12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="C12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="D12" t="str" cm="1">
-        <f t="array" ref="D12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="D12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="E12" t="str" cm="1">
-        <f t="array" ref="E12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="E12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="F12" t="str" cm="1">
-        <f t="array" ref="F12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="F12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="G12" t="str" cm="1">
-        <f t="array" ref="G12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="G12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="H12" t="str" cm="1">
-        <f t="array" ref="H12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="H12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="I12" t="str" cm="1">
-        <f t="array" ref="I12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="I12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="J12" t="str" cm="1">
-        <f t="array" ref="J12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="J12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="K12" t="str" cm="1">
-        <f t="array" ref="K12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="K12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="L12" t="str" cm="1">
-        <f t="array" ref="L12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="L12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M12" t="str" cm="1">
-        <f t="array" ref="M12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="M12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N12" t="str" cm="1">
-        <f t="array" ref="N12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="O12" t="str" cm="1">
-        <f t="array" ref="O12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P12" t="str" cm="1">
-        <f t="array" ref="P12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q12" t="str" cm="1">
-        <f t="array" ref="Q12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T12" t="s">
+        <f t="array" ref="N12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q12" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="T12" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>11</v>
       </c>
       <c r="B13" t="str" cm="1">
-        <f t="array" ref="B13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C13" t="str" cm="1">
+        <f t="array" ref="C13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D13" t="str" cm="1">
+        <f t="array" ref="D13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="E13" t="str" cm="1">
+        <f t="array" ref="E13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="F13" t="str" cm="1">
+        <f t="array" ref="F13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="G13" t="str" cm="1">
+        <f t="array" ref="G13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="H13" t="str" cm="1">
+        <f t="array" ref="H13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="I13" t="str" cm="1">
+        <f t="array" ref="I13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
-      <c r="C13" t="str" cm="1">
-        <f t="array" ref="C13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+      <c r="J13" t="str" cm="1">
+        <f t="array" ref="J13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
-      <c r="D13" t="str" cm="1">
-        <f t="array" ref="D13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+      <c r="K13" t="str" cm="1">
+        <f t="array" ref="K13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
-      <c r="E13" t="str" cm="1">
-        <f t="array" ref="E13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="F13" t="str" cm="1">
-        <f t="array" ref="F13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="G13" t="str" cm="1">
-        <f t="array" ref="G13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="H13" t="str" cm="1">
-        <f t="array" ref="H13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="I13" t="str" cm="1">
-        <f t="array" ref="I13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="J13" t="str" cm="1">
-        <f t="array" ref="J13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="K13" t="str" cm="1">
-        <f t="array" ref="K13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
       <c r="L13" t="str" cm="1">
-        <f t="array" ref="L13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="L13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M13" t="str" cm="1">
-        <f t="array" ref="M13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="M13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N13" t="str" cm="1">
-        <f t="array" ref="N13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="O13" t="str" cm="1">
-        <f t="array" ref="O13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P13" t="str" cm="1">
-        <f t="array" ref="P13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q13" t="str" cm="1">
-        <f t="array" ref="Q13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q13" t="s">
+        <v>42</v>
+      </c>
+      <c r="T13" s="9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>12</v>
       </c>
       <c r="B14" t="str" cm="1">
-        <f t="array" ref="B14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C14" t="str" cm="1">
-        <f t="array" ref="C14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D14" t="str" cm="1">
-        <f t="array" ref="D14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E14" t="str" cm="1">
-        <f t="array" ref="E14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F14" t="str" cm="1">
-        <f t="array" ref="F14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G14" t="str" cm="1">
-        <f t="array" ref="G14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H14" t="str" cm="1">
-        <f t="array" ref="H14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I14" t="str" cm="1">
-        <f t="array" ref="I14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="I14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="J14" t="str" cm="1">
-        <f t="array" ref="J14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="K14" t="str" cm="1">
-        <f t="array" ref="K14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="L14" t="str" cm="1">
-        <f t="array" ref="L14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="M14" t="str" cm="1">
-        <f t="array" ref="M14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="L14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
+      </c>
+      <c r="M14" t="s">
+        <v>50</v>
       </c>
       <c r="N14" t="str" cm="1">
-        <f t="array" ref="N14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="O14" t="str" cm="1">
-        <f t="array" ref="O14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P14" t="str" cm="1">
-        <f t="array" ref="P14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q14" t="str" cm="1">
-        <f t="array" ref="Q14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q14" t="s">
+        <v>42</v>
+      </c>
+      <c r="T14" s="9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>13</v>
       </c>
       <c r="B15" t="str" cm="1">
-        <f t="array" ref="B15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C15" t="str" cm="1">
-        <f t="array" ref="C15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D15" t="str" cm="1">
-        <f t="array" ref="D15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="E15" t="str" cm="1">
-        <f t="array" ref="E15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="F15" t="str" cm="1">
-        <f t="array" ref="F15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G15" t="str" cm="1">
-        <f t="array" ref="G15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H15" t="str" cm="1">
-        <f t="array" ref="H15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I15" t="str" cm="1">
-        <f t="array" ref="I15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="I15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="J15" t="str" cm="1">
-        <f t="array" ref="J15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="K15" t="str" cm="1">
-        <f t="array" ref="K15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="L15" t="str" cm="1">
-        <f t="array" ref="L15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="L15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M15" t="str" cm="1">
-        <f t="array" ref="M15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="M15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N15" t="str" cm="1">
-        <f t="array" ref="N15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="O15" t="str" cm="1">
-        <f t="array" ref="O15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Shifting cultivation</v>
-      </c>
-      <c r="P15" t="str" cm="1">
-        <f t="array" ref="P15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q15" t="str" cm="1">
-        <f t="array" ref="Q15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T15" t="s">
-        <v>50</v>
-      </c>
-      <c r="W15" s="9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q15" t="s">
+        <v>49</v>
+      </c>
+      <c r="T15" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>14</v>
       </c>
       <c r="B16" t="str" cm="1">
-        <f t="array" ref="B16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C16" t="str" cm="1">
-        <f t="array" ref="C16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D16" t="str" cm="1">
-        <f t="array" ref="D16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E16" t="str" cm="1">
-        <f t="array" ref="E16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="F16" t="str" cm="1">
-        <f t="array" ref="F16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G16" t="str" cm="1">
-        <f t="array" ref="G16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="H16" t="str" cm="1">
+        <f t="array" ref="H16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="I16" t="str" cm="1">
+        <f t="array" ref="I16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
-      <c r="H16" t="str" cm="1">
-        <f t="array" ref="H16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+      <c r="J16" t="str" cm="1">
+        <f t="array" ref="J16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
-      <c r="I16" t="str" cm="1">
-        <f t="array" ref="I16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="J16" t="str" cm="1">
-        <f t="array" ref="J16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
       <c r="K16" t="str" cm="1">
-        <f t="array" ref="K16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="L16" t="str" cm="1">
-        <f t="array" ref="L16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="L16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M16" t="str" cm="1">
-        <f t="array" ref="M16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="M16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N16" t="str" cm="1">
-        <f t="array" ref="N16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="O16" t="str" cm="1">
-        <f t="array" ref="O16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Shifting cultivation</v>
-      </c>
-      <c r="P16" t="str" cm="1">
-        <f t="array" ref="P16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q16" t="str" cm="1">
-        <f t="array" ref="Q16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T16" t="s">
-        <v>51</v>
-      </c>
-      <c r="W16" s="9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q16" t="s">
+        <v>47</v>
+      </c>
+      <c r="T16" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>15</v>
       </c>
       <c r="B17" t="str" cm="1">
-        <f t="array" ref="B17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="B17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="C17" t="str" cm="1">
-        <f t="array" ref="C17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="C17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="D17" t="str" cm="1">
-        <f t="array" ref="D17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E17" t="str" cm="1">
-        <f t="array" ref="E17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F17" t="str" cm="1">
-        <f t="array" ref="F17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G17" t="str" cm="1">
-        <f t="array" ref="G17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H17" t="str" cm="1">
-        <f t="array" ref="H17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="H17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="I17" t="str" cm="1">
-        <f t="array" ref="I17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="I17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="J17" t="str" cm="1">
-        <f t="array" ref="J17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K17" t="str" cm="1">
-        <f t="array" ref="K17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L17" t="str" cm="1">
-        <f t="array" ref="L17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="L17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M17" t="str" cm="1">
-        <f t="array" ref="M17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="M17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N17" t="str" cm="1">
-        <f t="array" ref="N17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="O17" t="str" cm="1">
-        <f t="array" ref="O17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Shifting cultivation</v>
-      </c>
-      <c r="P17" t="str" cm="1">
-        <f t="array" ref="P17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q17" t="str" cm="1">
-        <f t="array" ref="Q17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T17" t="s">
-        <v>46</v>
-      </c>
-      <c r="W17" s="9" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>16</v>
       </c>
       <c r="B18" t="str" cm="1">
-        <f t="array" ref="B18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="B18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="C18" t="str" cm="1">
-        <f t="array" ref="C18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="C18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="D18" t="str" cm="1">
-        <f t="array" ref="D18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E18" t="str" cm="1">
-        <f t="array" ref="E18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="F18" t="str" cm="1">
-        <f t="array" ref="F18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="G18" t="str" cm="1">
-        <f t="array" ref="G18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="G18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="H18" t="str" cm="1">
-        <f t="array" ref="H18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="H18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="I18" t="str" cm="1">
-        <f t="array" ref="I18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="I18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="J18" t="str" cm="1">
-        <f t="array" ref="J18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="K18" t="str" cm="1">
-        <f t="array" ref="K18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="L18" t="str" cm="1">
-        <f t="array" ref="L18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="L18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M18" t="str" cm="1">
-        <f t="array" ref="M18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="M18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N18" t="str" cm="1">
-        <f t="array" ref="N18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="O18" t="str" cm="1">
-        <f t="array" ref="O18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Shifting cultivation</v>
-      </c>
-      <c r="P18" t="str" cm="1">
-        <f t="array" ref="P18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q18" t="str" cm="1">
-        <f t="array" ref="Q18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T18" t="s">
-        <v>46</v>
-      </c>
-      <c r="W18" s="9" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>17</v>
       </c>
       <c r="B19" t="str" cm="1">
-        <f t="array" ref="B19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C19" t="str" cm="1">
-        <f t="array" ref="C19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="C19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="D19" t="str" cm="1">
-        <f t="array" ref="D19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E19" t="str" cm="1">
-        <f t="array" ref="E19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="E19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="F19" t="str" cm="1">
-        <f t="array" ref="F19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G19" t="str" cm="1">
-        <f t="array" ref="G19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H19" t="str" cm="1">
-        <f t="array" ref="H19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="H19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="I19" t="str" cm="1">
-        <f t="array" ref="I19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="I19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="J19" t="str" cm="1">
-        <f t="array" ref="J19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="J19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="K19" t="str" cm="1">
-        <f t="array" ref="K19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="K19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="L19" t="str" cm="1">
-        <f t="array" ref="L19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="L19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M19" t="str" cm="1">
-        <f t="array" ref="M19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="M19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N19" t="str" cm="1">
-        <f t="array" ref="N19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="O19" t="str" cm="1">
-        <f t="array" ref="O19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="P19" t="str" cm="1">
-        <f t="array" ref="P19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q19" t="str" cm="1">
-        <f t="array" ref="Q19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T19" t="s">
-        <v>55</v>
-      </c>
-      <c r="W19" s="9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>18</v>
       </c>
-      <c r="B20" t="str" cm="1">
-        <f t="array" ref="B20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="C20" t="str" cm="1">
-        <f t="array" ref="C20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="D20" t="str" cm="1">
-        <f t="array" ref="D20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="E20" t="str" cm="1">
-        <f t="array" ref="E20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="F20" t="str" cm="1">
-        <f t="array" ref="F20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="G20" t="str" cm="1">
-        <f t="array" ref="G20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="H20" t="str" cm="1">
-        <f t="array" ref="H20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="I20" t="str" cm="1">
-        <f t="array" ref="I20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="J20" t="str" cm="1">
-        <f t="array" ref="J20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="K20" t="str" cm="1">
-        <f t="array" ref="K20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+      <c r="B20" t="e" cm="1">
+        <f t="array" ref="B20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C20" t="e" cm="1">
+        <f t="array" ref="C20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D20" t="e" cm="1">
+        <f t="array" ref="D20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E20" t="e" cm="1">
+        <f t="array" ref="E20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F20" t="e" cm="1">
+        <f t="array" ref="F20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G20" t="e" cm="1">
+        <f t="array" ref="G20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H20" t="e" cm="1">
+        <f t="array" ref="H20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I20" t="e" cm="1">
+        <f t="array" ref="I20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J20" t="e" cm="1">
+        <f t="array" ref="J20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K20" t="e" cm="1">
+        <f t="array" ref="K20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
       </c>
       <c r="L20" t="str" cm="1">
-        <f t="array" ref="L20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, L$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="L20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M20" t="str" cm="1">
-        <f t="array" ref="M20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, M$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="M20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N20" t="str" cm="1">
-        <f t="array" ref="N20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, N$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="O20" t="str" cm="1">
-        <f t="array" ref="O20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$Q$19, O$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Shifting cultivation</v>
-      </c>
-      <c r="P20" t="str" cm="1">
-        <f t="array" ref="P20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$Q$19, P$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="Q20" t="str" cm="1">
-        <f t="array" ref="Q20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$Q$19, Q$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="T20" t="s">
-        <v>53</v>
-      </c>
-      <c r="W20" s="9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
+        <f t="array" ref="N20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B21" t="e" cm="1">
+        <f t="array" ref="B21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C21" t="e" cm="1">
+        <f t="array" ref="C21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D21" t="e" cm="1">
+        <f t="array" ref="D21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E21" t="e" cm="1">
+        <f t="array" ref="E21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F21" t="e" cm="1">
+        <f t="array" ref="F21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G21" t="e" cm="1">
+        <f t="array" ref="G21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H21" t="e" cm="1">
+        <f t="array" ref="H21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I21" t="e" cm="1">
+        <f t="array" ref="I21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J21" t="e" cm="1">
+        <f t="array" ref="J21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K21" t="e" cm="1">
+        <f t="array" ref="K21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L21" t="str" cm="1">
+        <f t="array" ref="L21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M21" t="str" cm="1">
+        <f t="array" ref="M21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="N21" t="str" cm="1">
+        <f t="array" ref="N21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="B22" t="e" cm="1">
+        <f t="array" ref="B22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C22" t="e" cm="1">
+        <f t="array" ref="C22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D22" t="e" cm="1">
+        <f t="array" ref="D22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E22" t="e" cm="1">
+        <f t="array" ref="E22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F22" t="e" cm="1">
+        <f t="array" ref="F22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G22" t="e" cm="1">
+        <f t="array" ref="G22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H22" t="e" cm="1">
+        <f t="array" ref="H22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I22" t="e" cm="1">
+        <f t="array" ref="I22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J22" t="e" cm="1">
+        <f t="array" ref="J22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K22" t="e" cm="1">
+        <f t="array" ref="K22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L22" t="str" cm="1">
+        <f t="array" ref="L22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M22" t="str" cm="1">
+        <f t="array" ref="M22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="N22" t="str" cm="1">
+        <f t="array" ref="N22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A24" s="8">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A25" s="8">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A26" s="8">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A27" s="8">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A28" s="8">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A29" s="8">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A30" s="8">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A31" s="8">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A32" s="8">
-        <v>30</v>
-      </c>
+      <c r="B23" t="e" cm="1">
+        <f t="array" ref="B23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C23" t="e" cm="1">
+        <f t="array" ref="C23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D23" t="e" cm="1">
+        <f t="array" ref="D23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E23" t="e" cm="1">
+        <f t="array" ref="E23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F23" t="e" cm="1">
+        <f t="array" ref="F23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G23" t="e" cm="1">
+        <f t="array" ref="G23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H23" t="e" cm="1">
+        <f t="array" ref="H23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I23" t="e" cm="1">
+        <f t="array" ref="I23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J23" t="e" cm="1">
+        <f t="array" ref="J23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K23" t="e" cm="1">
+        <f t="array" ref="K23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L23" t="str" cm="1">
+        <f t="array" ref="L23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M23" t="str" cm="1">
+        <f t="array" ref="M23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="N23" t="str" cm="1">
+        <f t="array" ref="N23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A24" s="8"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A25" s="8"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" s="8"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" s="8"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A28" s="8"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A29" s="8"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A30" s="8"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A31" s="8"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A32" s="8"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" s="8">
-        <v>31</v>
-      </c>
+      <c r="A33" s="8"/>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8">
-        <v>32</v>
-      </c>
+      <c r="A34" s="8"/>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" s="8">
-        <v>33</v>
-      </c>
+      <c r="A35" s="8"/>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" s="8">
-        <v>34</v>
-      </c>
+      <c r="A36" s="8"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8">
-        <v>35</v>
-      </c>
+      <c r="A37" s="8"/>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8">
-        <v>36</v>
-      </c>
+      <c r="A38" s="8"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" s="8">
-        <v>37</v>
-      </c>
+      <c r="A39" s="8"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" s="8">
-        <v>38</v>
-      </c>
+      <c r="A40" s="8"/>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A41" s="8">
-        <v>39</v>
-      </c>
+      <c r="A41" s="8"/>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A42" s="8">
-        <v>40</v>
-      </c>
+      <c r="A42" s="8"/>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" s="8">
-        <v>41</v>
-      </c>
+      <c r="A43" s="8"/>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="8">
-        <v>42</v>
-      </c>
+      <c r="A44" s="8"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" s="8">
-        <v>43</v>
-      </c>
+      <c r="A45" s="8"/>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" s="8">
-        <v>44</v>
-      </c>
+      <c r="A46" s="8"/>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="8">
-        <v>45</v>
-      </c>
+      <c r="A47" s="8"/>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="8">
-        <v>46</v>
-      </c>
+      <c r="A48" s="8"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="8">
-        <v>47</v>
-      </c>
+      <c r="A49" s="8"/>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="8">
-        <v>48</v>
-      </c>
+      <c r="A50" s="8"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="8">
-        <v>49</v>
-      </c>
+      <c r="A51" s="8"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="8">
-        <v>50</v>
-      </c>
+      <c r="A52" s="8"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
@@ -3191,20 +2783,8 @@
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" s="8"/>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A66" s="8"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A67" s="8"/>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A68" s="8"/>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A69" s="8"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:T1 B2:N1048576">
+  <conditionalFormatting sqref="B1:Q1 B2:K1048576">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"short veg"</formula>
     </cfRule>
@@ -3212,7 +2792,7 @@
       <formula>"tall veg"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1:N1048576">
+  <conditionalFormatting sqref="L1:N1 B1:K1048576">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"cropland"</formula>
     </cfRule>

</xml_diff>

<commit_message>
LC -> LU conversion: - Updated shifting cultivation
</commit_message>
<xml_diff>
--- a/src/LULUCF/scripts/postprocessing/conversion_LUC_scenarios.xlsx
+++ b/src/LULUCF/scripts/postprocessing/conversion_LUC_scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\scripts\postprocessing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47FE53F1-2657-48F1-87CE-4B36D5CA164A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9837866C-F0CA-4217-9EAB-030630691D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="54">
   <si>
     <t>Driver</t>
   </si>
@@ -177,12 +177,6 @@
     <t xml:space="preserve">Expected result: </t>
   </si>
   <si>
-    <t>After tall vegetation is established, short veg is considered forest since SDPT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forest the entire time series because logging concession </t>
-  </si>
-  <si>
     <t>Forest remaining forest</t>
   </si>
   <si>
@@ -192,28 +186,43 @@
     <t>Cropland remaining cropland</t>
   </si>
   <si>
-    <t>Forest remaining forest (if n_years_unstocked_forest = 5)</t>
+    <t xml:space="preserve">Forest remaining forest </t>
+  </si>
+  <si>
+    <t>or cropland remaining cropland</t>
+  </si>
+  <si>
+    <t>Forest remaining forest (logging concessions)</t>
+  </si>
+  <si>
+    <t>Forest remaining forest (SDPT planted fprest)</t>
+  </si>
+  <si>
+    <t>Forest remaining forest (n_years_unstocked_forest &lt;= 3)</t>
+  </si>
+  <si>
+    <t>Forest land to grassland in 2017</t>
+  </si>
+  <si>
+    <t>Forest remaining forest (logging driver, initial years)</t>
+  </si>
+  <si>
+    <t>Forest remaining forest (logging driver, teminal years)</t>
   </si>
   <si>
     <t>Forest to cropland in 2022</t>
   </si>
   <si>
-    <t>Forest to cropland in 2017</t>
-  </si>
-  <si>
-    <t>not conversion (shifting ag)???</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forest remaining forest </t>
-  </si>
-  <si>
-    <t>or cropland remaining cropland</t>
-  </si>
-  <si>
-    <t>Back and foth between Forest and cropland until 2018?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">* </t>
+    <t>or should this be cropland remaining cropland</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Forest to cropland in 2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forest to cropland in 2017 </t>
   </si>
 </sst>
 </file>
@@ -612,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="8"/>
@@ -739,7 +748,7 @@
         <v>1</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -852,13 +861,13 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -873,13 +882,13 @@
         <v>1</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L7">
         <v>4</v>
@@ -896,7 +905,7 @@
         <v>3</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -918,113 +927,115 @@
       </c>
       <c r="K8">
         <v>1</v>
+      </c>
+      <c r="L8">
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>8</v>
       </c>
-      <c r="B9" s="1">
-        <v>7</v>
-      </c>
-      <c r="C9" s="1">
-        <v>7</v>
-      </c>
-      <c r="D9" s="1">
-        <v>7</v>
-      </c>
-      <c r="E9" s="1">
-        <v>7</v>
-      </c>
-      <c r="F9" s="1">
-        <v>7</v>
-      </c>
-      <c r="G9" s="1">
-        <v>7</v>
-      </c>
-      <c r="H9" s="1">
-        <v>7</v>
-      </c>
-      <c r="I9" s="1">
-        <v>7</v>
-      </c>
-      <c r="J9" s="1">
-        <v>7</v>
-      </c>
-      <c r="K9" s="1">
-        <v>7</v>
-      </c>
-      <c r="L9" s="6"/>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>9</v>
       </c>
       <c r="B10" s="1">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1">
+        <v>7</v>
+      </c>
+      <c r="D10" s="1">
+        <v>7</v>
+      </c>
+      <c r="E10" s="1">
+        <v>7</v>
+      </c>
+      <c r="F10" s="1">
+        <v>7</v>
+      </c>
+      <c r="G10" s="1">
+        <v>7</v>
+      </c>
+      <c r="H10" s="1">
+        <v>7</v>
+      </c>
+      <c r="I10" s="1">
+        <v>7</v>
+      </c>
+      <c r="J10" s="1">
+        <v>7</v>
+      </c>
+      <c r="K10" s="1">
+        <v>7</v>
+      </c>
+      <c r="L10" s="6"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11" s="8">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
         <v>5</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C11" s="1">
         <v>5</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D11" s="1">
         <v>5</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E11" s="1">
         <v>5</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F11" s="1">
         <v>5</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G11" s="1">
         <v>5</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H11" s="1">
         <v>5</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I11" s="1">
         <v>5</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J11" s="1">
         <v>5</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K11" s="1">
         <v>5</v>
-      </c>
-      <c r="L10" s="6"/>
-    </row>
-    <row r="11" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1">
-        <v>10</v>
-      </c>
-      <c r="C11" s="1">
-        <v>10</v>
-      </c>
-      <c r="D11" s="1">
-        <v>10</v>
-      </c>
-      <c r="E11" s="1">
-        <v>10</v>
-      </c>
-      <c r="F11" s="1">
-        <v>10</v>
-      </c>
-      <c r="G11" s="1">
-        <v>10</v>
-      </c>
-      <c r="H11" s="1">
-        <v>10</v>
-      </c>
-      <c r="I11" s="1">
-        <v>10</v>
-      </c>
-      <c r="J11" s="1">
-        <v>10</v>
-      </c>
-      <c r="K11" s="1">
-        <v>10</v>
       </c>
       <c r="L11" s="6"/>
     </row>
@@ -1033,25 +1044,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C12" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D12" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E12" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F12" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G12" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H12" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I12" s="1">
         <v>10</v>
@@ -1062,7 +1073,7 @@
       <c r="K12" s="1">
         <v>10</v>
       </c>
-      <c r="L12" s="7"/>
+      <c r="L12" s="6"/>
     </row>
     <row r="13" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
@@ -1098,9 +1109,7 @@
       <c r="K13" s="1">
         <v>10</v>
       </c>
-      <c r="L13" s="7">
-        <v>3</v>
-      </c>
+      <c r="L13" s="7"/>
     </row>
     <row r="14" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
@@ -1113,10 +1122,10 @@
         <v>7</v>
       </c>
       <c r="D14" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E14" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F14" s="1">
         <v>7</v>
@@ -1151,7 +1160,7 @@
         <v>7</v>
       </c>
       <c r="D15" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E15" s="1">
         <v>10</v>
@@ -1192,7 +1201,7 @@
         <v>7</v>
       </c>
       <c r="E16" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F16" s="1">
         <v>7</v>
@@ -1204,24 +1213,24 @@
         <v>7</v>
       </c>
       <c r="I16" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J16" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K16" s="1">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L16" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>16</v>
       </c>
       <c r="B17" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C17" s="1">
         <v>7</v>
@@ -1230,34 +1239,36 @@
         <v>7</v>
       </c>
       <c r="E17" s="1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F17" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G17" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H17" s="1">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I17" s="1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J17" s="1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K17" s="1">
-        <v>10</v>
-      </c>
-      <c r="L17" s="7"/>
+        <v>5</v>
+      </c>
+      <c r="L17" s="7">
+        <v>3</v>
+      </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>17</v>
       </c>
       <c r="B18" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C18" s="1">
         <v>7</v>
@@ -1266,27 +1277,63 @@
         <v>7</v>
       </c>
       <c r="E18" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F18" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G18" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H18" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I18" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J18" s="1">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K18" s="1">
-        <v>7</v>
-      </c>
-      <c r="L18" s="7">
+        <v>10</v>
+      </c>
+      <c r="L18" s="7"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" s="8">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1">
+        <v>7</v>
+      </c>
+      <c r="C19" s="1">
+        <v>7</v>
+      </c>
+      <c r="D19" s="1">
+        <v>7</v>
+      </c>
+      <c r="E19" s="1">
+        <v>7</v>
+      </c>
+      <c r="F19" s="1">
+        <v>7</v>
+      </c>
+      <c r="G19" s="1">
+        <v>7</v>
+      </c>
+      <c r="H19" s="1">
+        <v>7</v>
+      </c>
+      <c r="I19" s="1">
+        <v>7</v>
+      </c>
+      <c r="J19" s="1">
+        <v>7</v>
+      </c>
+      <c r="K19" s="1">
+        <v>7</v>
+      </c>
+      <c r="L19" s="7">
         <v>3</v>
       </c>
     </row>
@@ -1297,7 +1344,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FD5E73A-BF21-4771-A2AF-1B9A394A8B1D}">
-  <dimension ref="A1:T65"/>
+  <dimension ref="A1:T66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="12" max="12" width="20.5546875" bestFit="1" customWidth="1"/>
@@ -1406,55 +1453,55 @@
         <v>1</v>
       </c>
       <c r="B3" t="str" cm="1">
-        <f t="array" ref="B3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="C3" t="str" cm="1">
-        <f t="array" ref="C3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D3" t="str" cm="1">
-        <f t="array" ref="D3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E3" t="str" cm="1">
-        <f t="array" ref="E3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F3" t="str" cm="1">
-        <f t="array" ref="F3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G3" t="str" cm="1">
-        <f t="array" ref="G3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H3" t="str" cm="1">
-        <f t="array" ref="H3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I3" t="str" cm="1">
-        <f t="array" ref="I3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J3" t="str" cm="1">
-        <f t="array" ref="J3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="K3" t="str" cm="1">
-        <f t="array" ref="K3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L3" t="str" cm="1">
-        <f t="array" ref="L3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M3" t="str" cm="1">
-        <f t="array" ref="M3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N3" t="str" cm="1">
-        <f t="array" ref="N3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v>yes</v>
       </c>
       <c r="Q3" t="s">
@@ -1466,59 +1513,59 @@
         <v>2</v>
       </c>
       <c r="B4" t="str" cm="1">
-        <f t="array" ref="B4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="C4" t="str" cm="1">
-        <f t="array" ref="C4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D4" t="str" cm="1">
-        <f t="array" ref="D4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E4" t="str" cm="1">
-        <f t="array" ref="E4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F4" t="str" cm="1">
-        <f t="array" ref="F4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G4" t="str" cm="1">
-        <f t="array" ref="G4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H4" t="str" cm="1">
-        <f t="array" ref="H4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I4" t="str" cm="1">
-        <f t="array" ref="I4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J4" t="str" cm="1">
-        <f t="array" ref="J4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="K4" t="str" cm="1">
-        <f t="array" ref="K4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L4" t="str" cm="1">
-        <f t="array" ref="L4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M4" t="str" cm="1">
-        <f t="array" ref="M4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v>wood fiber</v>
+        <f t="array" ref="M4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v>oil palm</v>
       </c>
       <c r="N4" t="str" cm="1">
-        <f t="array" ref="N4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
@@ -1526,59 +1573,59 @@
         <v>3</v>
       </c>
       <c r="B5" t="str" cm="1">
-        <f t="array" ref="B5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="C5" t="str" cm="1">
-        <f t="array" ref="C5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D5" t="str" cm="1">
-        <f t="array" ref="D5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E5" t="str" cm="1">
-        <f t="array" ref="E5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F5" t="str" cm="1">
-        <f t="array" ref="F5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G5" t="str" cm="1">
-        <f t="array" ref="G5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H5" t="str" cm="1">
-        <f t="array" ref="H5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I5" t="str" cm="1">
-        <f t="array" ref="I5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="J5" t="str" cm="1">
-        <f t="array" ref="J5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="K5" t="str" cm="1">
-        <f t="array" ref="K5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="L5" t="str" cm="1">
-        <f t="array" ref="L5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M5" t="str" cm="1">
-        <f t="array" ref="M5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N5" t="str" cm="1">
-        <f t="array" ref="N5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q5" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
@@ -1586,59 +1633,59 @@
         <v>4</v>
       </c>
       <c r="B6" t="str" cm="1">
-        <f t="array" ref="B6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C6" t="str" cm="1">
-        <f t="array" ref="C6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D6" t="str" cm="1">
-        <f t="array" ref="D6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E6" t="str" cm="1">
-        <f t="array" ref="E6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F6" t="str" cm="1">
-        <f t="array" ref="F6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G6" t="str" cm="1">
-        <f t="array" ref="G6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H6" t="str" cm="1">
-        <f t="array" ref="H6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I6" t="str" cm="1">
-        <f t="array" ref="I6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J6" t="str" cm="1">
-        <f t="array" ref="J6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K6" t="str" cm="1">
-        <f t="array" ref="K6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L6" t="str" cm="1">
-        <f t="array" ref="L6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M6" t="str" cm="1">
-        <f t="array" ref="M6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N6" t="str" cm="1">
-        <f t="array" ref="N6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q6" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.3">
@@ -1646,59 +1693,59 @@
         <v>5</v>
       </c>
       <c r="B7" t="str" cm="1">
-        <f t="array" ref="B7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C7" t="str" cm="1">
-        <f t="array" ref="C7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D7" t="str" cm="1">
-        <f t="array" ref="D7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E7" t="str" cm="1">
-        <f t="array" ref="E7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F7" t="str" cm="1">
-        <f t="array" ref="F7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G7" t="str" cm="1">
-        <f t="array" ref="G7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H7" t="str" cm="1">
-        <f t="array" ref="H7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I7" t="str" cm="1">
-        <f t="array" ref="I7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J7" t="str" cm="1">
-        <f t="array" ref="J7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K7" t="str" cm="1">
-        <f t="array" ref="K7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L7" t="str" cm="1">
-        <f t="array" ref="L7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M7" t="str" cm="1">
-        <f t="array" ref="M7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N7" t="str" cm="1">
-        <f t="array" ref="N7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
@@ -1706,59 +1753,59 @@
         <v>6</v>
       </c>
       <c r="B8" t="str" cm="1">
-        <f t="array" ref="B8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="B8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="C8" t="str" cm="1">
-        <f t="array" ref="C8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="C8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="D8" t="str" cm="1">
-        <f t="array" ref="D8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="E8" t="str" cm="1">
-        <f t="array" ref="E8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F8" t="str" cm="1">
-        <f t="array" ref="F8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G8" t="str" cm="1">
-        <f t="array" ref="G8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H8" t="str" cm="1">
-        <f t="array" ref="H8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I8" t="str" cm="1">
-        <f t="array" ref="I8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="I8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="J8" t="str" cm="1">
-        <f t="array" ref="J8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="J8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="K8" t="str" cm="1">
-        <f t="array" ref="K8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="K8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="L8" t="str" cm="1">
-        <f t="array" ref="L8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Logging</v>
       </c>
       <c r="M8" t="str" cm="1">
-        <f t="array" ref="M8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N8" t="str" cm="1">
-        <f t="array" ref="N8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q8" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
@@ -1766,59 +1813,59 @@
         <v>7</v>
       </c>
       <c r="B9" t="str" cm="1">
-        <f t="array" ref="B9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C9" t="str" cm="1">
-        <f t="array" ref="C9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D9" t="str" cm="1">
-        <f t="array" ref="D9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="D9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="E9" t="str" cm="1">
-        <f t="array" ref="E9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F9" t="str" cm="1">
-        <f t="array" ref="F9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G9" t="str" cm="1">
-        <f t="array" ref="G9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H9" t="str" cm="1">
-        <f t="array" ref="H9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I9" t="str" cm="1">
-        <f t="array" ref="I9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J9" t="str" cm="1">
-        <f t="array" ref="J9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="K9" t="str" cm="1">
-        <f t="array" ref="K9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L9" t="str" cm="1">
-        <f t="array" ref="L9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
+        <f t="array" ref="L9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Logging</v>
       </c>
       <c r="M9" t="str" cm="1">
-        <f t="array" ref="M9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N9" t="str" cm="1">
-        <f t="array" ref="N9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q9" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
@@ -1826,59 +1873,59 @@
         <v>8</v>
       </c>
       <c r="B10" t="str" cm="1">
-        <f t="array" ref="B10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C10" t="str" cm="1">
-        <f t="array" ref="C10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D10" t="str" cm="1">
-        <f t="array" ref="D10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="E10" t="str" cm="1">
-        <f t="array" ref="E10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F10" t="str" cm="1">
-        <f t="array" ref="F10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="G10" t="str" cm="1">
-        <f t="array" ref="G10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="G10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="H10" t="str" cm="1">
-        <f t="array" ref="H10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="H10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="I10" t="str" cm="1">
-        <f t="array" ref="I10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="I10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="J10" t="str" cm="1">
-        <f t="array" ref="J10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K10" t="str" cm="1">
-        <f t="array" ref="K10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L10" t="str" cm="1">
-        <f t="array" ref="L10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M10" t="str" cm="1">
-        <f t="array" ref="M10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N10" t="str" cm="1">
-        <f t="array" ref="N10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
@@ -1886,62 +1933,59 @@
         <v>9</v>
       </c>
       <c r="B11" t="str" cm="1">
-        <f t="array" ref="B11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="B11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="C11" t="str" cm="1">
-        <f t="array" ref="C11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="C11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="D11" t="str" cm="1">
-        <f t="array" ref="D11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="D11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="E11" t="str" cm="1">
-        <f t="array" ref="E11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="E11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="F11" t="str" cm="1">
-        <f t="array" ref="F11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="F11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="G11" t="str" cm="1">
-        <f t="array" ref="G11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="G11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="H11" t="str" cm="1">
-        <f t="array" ref="H11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="H11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="I11" t="str" cm="1">
-        <f t="array" ref="I11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="I11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="J11" t="str" cm="1">
-        <f t="array" ref="J11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="J11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="K11" t="str" cm="1">
-        <f t="array" ref="K11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="K11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="L11" t="str" cm="1">
-        <f t="array" ref="L11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M11" t="str" cm="1">
-        <f t="array" ref="M11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N11" t="str" cm="1">
-        <f t="array" ref="N11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q11" t="s">
-        <v>44</v>
-      </c>
-      <c r="T11" s="9" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
@@ -1949,187 +1993,181 @@
         <v>10</v>
       </c>
       <c r="B12" t="str" cm="1">
-        <f t="array" ref="B12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="B12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="C12" t="str" cm="1">
-        <f t="array" ref="C12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="C12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="D12" t="str" cm="1">
-        <f t="array" ref="D12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="D12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="E12" t="str" cm="1">
-        <f t="array" ref="E12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="E12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F12" t="str" cm="1">
-        <f t="array" ref="F12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="F12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="G12" t="str" cm="1">
-        <f t="array" ref="G12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="G12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="H12" t="str" cm="1">
-        <f t="array" ref="H12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="H12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="I12" t="str" cm="1">
-        <f t="array" ref="I12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="I12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="J12" t="str" cm="1">
-        <f t="array" ref="J12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="J12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K12" t="str" cm="1">
-        <f t="array" ref="K12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="K12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L12" t="str" cm="1">
-        <f t="array" ref="L12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M12" t="str" cm="1">
-        <f t="array" ref="M12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N12" t="str" cm="1">
-        <f t="array" ref="N12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q12" t="s">
-        <v>45</v>
-      </c>
-      <c r="T12" s="9" t="s">
-        <v>46</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="T12" s="9"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>11</v>
       </c>
       <c r="B13" t="str" cm="1">
-        <f t="array" ref="B13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="B13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="C13" t="str" cm="1">
-        <f t="array" ref="C13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="C13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="D13" t="str" cm="1">
-        <f t="array" ref="D13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="E13" t="str" cm="1">
-        <f t="array" ref="E13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="F13" t="str" cm="1">
-        <f t="array" ref="F13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="G13" t="str" cm="1">
-        <f t="array" ref="G13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="G13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="H13" t="str" cm="1">
-        <f t="array" ref="H13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="H13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="I13" t="str" cm="1">
-        <f t="array" ref="I13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J13" t="str" cm="1">
-        <f t="array" ref="J13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K13" t="str" cm="1">
-        <f t="array" ref="K13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L13" t="str" cm="1">
-        <f t="array" ref="L13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M13" t="str" cm="1">
-        <f t="array" ref="M13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N13" t="str" cm="1">
-        <f t="array" ref="N13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q13" t="s">
-        <v>42</v>
-      </c>
-      <c r="T13" s="9" t="s">
-        <v>2</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="T13" s="9"/>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>12</v>
       </c>
       <c r="B14" t="str" cm="1">
-        <f t="array" ref="B14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C14" t="str" cm="1">
-        <f t="array" ref="C14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D14" t="str" cm="1">
-        <f t="array" ref="D14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E14" t="str" cm="1">
-        <f t="array" ref="E14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F14" t="str" cm="1">
-        <f t="array" ref="F14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G14" t="str" cm="1">
-        <f t="array" ref="G14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H14" t="str" cm="1">
-        <f t="array" ref="H14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I14" t="str" cm="1">
-        <f t="array" ref="I14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J14" t="str" cm="1">
-        <f t="array" ref="J14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K14" t="str" cm="1">
-        <f t="array" ref="K14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L14" t="str" cm="1">
-        <f t="array" ref="L14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Shifting cultivation</v>
-      </c>
-      <c r="M14" t="s">
-        <v>50</v>
+        <f t="array" ref="L14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M14" t="str" cm="1">
+        <f t="array" ref="M14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
       </c>
       <c r="N14" t="str" cm="1">
-        <f t="array" ref="N14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q14" t="s">
-        <v>42</v>
-      </c>
-      <c r="T14" s="9" t="s">
-        <v>2</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.3">
@@ -2137,62 +2175,62 @@
         <v>13</v>
       </c>
       <c r="B15" t="str" cm="1">
-        <f t="array" ref="B15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C15" t="str" cm="1">
-        <f t="array" ref="C15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D15" t="str" cm="1">
-        <f t="array" ref="D15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="E15" t="str" cm="1">
+        <f t="array" ref="E15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="F15" t="str" cm="1">
+        <f t="array" ref="F15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="G15" t="str" cm="1">
+        <f t="array" ref="G15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="H15" t="str" cm="1">
+        <f t="array" ref="H15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="I15" t="str" cm="1">
+        <f t="array" ref="I15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
-      <c r="E15" t="str" cm="1">
-        <f t="array" ref="E15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+      <c r="J15" t="str" cm="1">
+        <f t="array" ref="J15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
-      <c r="F15" t="str" cm="1">
-        <f t="array" ref="F15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="G15" t="str" cm="1">
-        <f t="array" ref="G15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="H15" t="str" cm="1">
-        <f t="array" ref="H15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="I15" t="str" cm="1">
-        <f t="array" ref="I15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+      <c r="K15" t="str" cm="1">
+        <f t="array" ref="K15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
-      <c r="J15" t="str" cm="1">
-        <f t="array" ref="J15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
-      <c r="K15" t="str" cm="1">
-        <f t="array" ref="K15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
-      </c>
       <c r="L15" t="str" cm="1">
-        <f t="array" ref="L15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Shifting cultivation</v>
       </c>
       <c r="M15" t="str" cm="1">
-        <f t="array" ref="M15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N15" t="str" cm="1">
-        <f t="array" ref="N15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q15" t="s">
         <v>49</v>
       </c>
-      <c r="T15" s="9" t="s">
-        <v>8</v>
+      <c r="T15" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
@@ -2200,488 +2238,567 @@
         <v>14</v>
       </c>
       <c r="B16" t="str" cm="1">
-        <f t="array" ref="B16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C16" t="str" cm="1">
-        <f t="array" ref="C16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D16" t="str" cm="1">
-        <f t="array" ref="D16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="D16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="E16" t="str" cm="1">
-        <f t="array" ref="E16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="F16" t="str" cm="1">
-        <f t="array" ref="F16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G16" t="str" cm="1">
-        <f t="array" ref="G16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H16" t="str" cm="1">
-        <f t="array" ref="H16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I16" t="str" cm="1">
-        <f t="array" ref="I16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J16" t="str" cm="1">
-        <f t="array" ref="J16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K16" t="str" cm="1">
-        <f t="array" ref="K16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L16" t="str" cm="1">
-        <f t="array" ref="L16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Shifting cultivation</v>
       </c>
       <c r="M16" t="str" cm="1">
-        <f t="array" ref="M16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N16" t="str" cm="1">
-        <f t="array" ref="N16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
         <v/>
       </c>
       <c r="Q16" t="s">
-        <v>47</v>
-      </c>
-      <c r="T16" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>15</v>
       </c>
       <c r="B17" t="str" cm="1">
-        <f t="array" ref="B17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C17" t="str" cm="1">
-        <f t="array" ref="C17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D17" t="str" cm="1">
-        <f t="array" ref="D17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E17" t="str" cm="1">
-        <f t="array" ref="E17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="E17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="F17" t="str" cm="1">
-        <f t="array" ref="F17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G17" t="str" cm="1">
-        <f t="array" ref="G17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H17" t="str" cm="1">
-        <f t="array" ref="H17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I17" t="str" cm="1">
-        <f t="array" ref="I17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="I17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="J17" t="str" cm="1">
-        <f t="array" ref="J17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="J17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="K17" t="str" cm="1">
-        <f t="array" ref="K17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
+        <f t="array" ref="K17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="L17" t="str" cm="1">
-        <f t="array" ref="L17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Shifting cultivation</v>
       </c>
       <c r="M17" t="str" cm="1">
-        <f t="array" ref="M17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N17" t="str" cm="1">
-        <f t="array" ref="N17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="array" ref="N17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q17" t="s">
+        <v>52</v>
+      </c>
+      <c r="T17" s="9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>16</v>
       </c>
       <c r="B18" t="str" cm="1">
-        <f t="array" ref="B18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="B18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="C18" t="str" cm="1">
-        <f t="array" ref="C18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D18" t="str" cm="1">
-        <f t="array" ref="D18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E18" t="str" cm="1">
-        <f t="array" ref="E18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="E18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="F18" t="str" cm="1">
-        <f t="array" ref="F18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="F18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="G18" t="str" cm="1">
-        <f t="array" ref="G18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="G18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="H18" t="str" cm="1">
-        <f t="array" ref="H18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="H18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="I18" t="str" cm="1">
-        <f t="array" ref="I18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="I18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="J18" t="str" cm="1">
-        <f t="array" ref="J18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="J18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="K18" t="str" cm="1">
-        <f t="array" ref="K18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>cropland</v>
+        <f t="array" ref="K18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L18" t="str" cm="1">
-        <f t="array" ref="L18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
+        <f t="array" ref="L18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M18" t="str" cm="1">
-        <f t="array" ref="M18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N18" t="str" cm="1">
-        <f t="array" ref="N18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="array" ref="N18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="P18" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>52</v>
+      </c>
+      <c r="T18" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>17</v>
       </c>
       <c r="B19" t="str" cm="1">
-        <f t="array" ref="B19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="B19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="C19" t="str" cm="1">
-        <f t="array" ref="C19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D19" t="str" cm="1">
-        <f t="array" ref="D19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E19" t="str" cm="1">
-        <f t="array" ref="E19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="E19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="F19" t="str" cm="1">
-        <f t="array" ref="F19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="F19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="G19" t="str" cm="1">
-        <f t="array" ref="G19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="G19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="H19" t="str" cm="1">
-        <f t="array" ref="H19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="H19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="I19" t="str" cm="1">
-        <f t="array" ref="I19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="I19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="J19" t="str" cm="1">
-        <f t="array" ref="J19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="J19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="K19" t="str" cm="1">
-        <f t="array" ref="K19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
+        <f t="array" ref="K19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>cropland</v>
       </c>
       <c r="L19" t="str" cm="1">
-        <f t="array" ref="L19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Shifting cultivation</v>
+        <f t="array" ref="L19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
       </c>
       <c r="M19" t="str" cm="1">
-        <f t="array" ref="M19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N19" t="str" cm="1">
-        <f t="array" ref="N19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="array" ref="N19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="Q19" t="s">
+        <v>40</v>
+      </c>
+      <c r="T19" s="9"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>18</v>
       </c>
-      <c r="B20" t="e" cm="1">
-        <f t="array" ref="B20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="C20" t="e" cm="1">
-        <f t="array" ref="C20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D20" t="e" cm="1">
-        <f t="array" ref="D20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E20" t="e" cm="1">
-        <f t="array" ref="E20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F20" t="e" cm="1">
-        <f t="array" ref="F20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G20" t="e" cm="1">
-        <f t="array" ref="G20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H20" t="e" cm="1">
-        <f t="array" ref="H20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="I20" t="e" cm="1">
-        <f t="array" ref="I20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="J20" t="e" cm="1">
-        <f t="array" ref="J20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K20" t="e" cm="1">
-        <f t="array" ref="K20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
+      <c r="B20" t="str" cm="1">
+        <f t="array" ref="B20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C20" t="str" cm="1">
+        <f t="array" ref="C20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D20" t="str" cm="1">
+        <f t="array" ref="D20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="E20" t="str" cm="1">
+        <f t="array" ref="E20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="F20" t="str" cm="1">
+        <f t="array" ref="F20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="G20" t="str" cm="1">
+        <f t="array" ref="G20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="H20" t="str" cm="1">
+        <f t="array" ref="H20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="I20" t="str" cm="1">
+        <f t="array" ref="I20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="J20" t="str" cm="1">
+        <f t="array" ref="J20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="K20" t="str" cm="1">
+        <f t="array" ref="K20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
       </c>
       <c r="L20" t="str" cm="1">
-        <f t="array" ref="L20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
+        <f t="array" ref="L20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M20" t="str" cm="1">
-        <f t="array" ref="M20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N20" t="str" cm="1">
-        <f t="array" ref="N20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="array" ref="N20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="P20" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>41</v>
+      </c>
+      <c r="T20" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
         <v>19</v>
       </c>
       <c r="B21" t="e" cm="1">
-        <f t="array" ref="B21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="C21" t="e" cm="1">
-        <f t="array" ref="C21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="D21" t="e" cm="1">
-        <f t="array" ref="D21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="E21" t="e" cm="1">
-        <f t="array" ref="E21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="F21" t="e" cm="1">
-        <f t="array" ref="F21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="G21" t="e" cm="1">
-        <f t="array" ref="G21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="H21" t="e" cm="1">
-        <f t="array" ref="H21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="I21" t="e" cm="1">
-        <f t="array" ref="I21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="J21" t="e" cm="1">
-        <f t="array" ref="J21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="K21" t="e" cm="1">
-        <f t="array" ref="K21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="L21" t="str" cm="1">
-        <f t="array" ref="L21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M21" t="str" cm="1">
-        <f t="array" ref="M21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N21" t="str" cm="1">
-        <f t="array" ref="N21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="array" ref="N21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>20</v>
       </c>
       <c r="B22" t="e" cm="1">
-        <f t="array" ref="B22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="C22" t="e" cm="1">
-        <f t="array" ref="C22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="D22" t="e" cm="1">
-        <f t="array" ref="D22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="E22" t="e" cm="1">
-        <f t="array" ref="E22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="F22" t="e" cm="1">
-        <f t="array" ref="F22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="G22" t="e" cm="1">
-        <f t="array" ref="G22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="H22" t="e" cm="1">
-        <f t="array" ref="H22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="I22" t="e" cm="1">
-        <f t="array" ref="I22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="J22" t="e" cm="1">
-        <f t="array" ref="J22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="K22" t="e" cm="1">
-        <f t="array" ref="K22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="L22" t="str" cm="1">
-        <f t="array" ref="L22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M22" t="str" cm="1">
-        <f t="array" ref="M22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N22" t="str" cm="1">
-        <f t="array" ref="N22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="array" ref="N22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
         <v>21</v>
       </c>
       <c r="B23" t="e" cm="1">
-        <f t="array" ref="B23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="C23" t="e" cm="1">
-        <f t="array" ref="C23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="D23" t="e" cm="1">
-        <f t="array" ref="D23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="E23" t="e" cm="1">
-        <f t="array" ref="E23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="F23" t="e" cm="1">
-        <f t="array" ref="F23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="G23" t="e" cm="1">
-        <f t="array" ref="G23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="H23" t="e" cm="1">
-        <f t="array" ref="H23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="I23" t="e" cm="1">
-        <f t="array" ref="I23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="J23" t="e" cm="1">
-        <f t="array" ref="J23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="K23" t="e" cm="1">
-        <f t="array" ref="K23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$18, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>#N/A</v>
       </c>
       <c r="L23" t="str" cm="1">
-        <f t="array" ref="L23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$18, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M23" t="str" cm="1">
-        <f t="array" ref="M23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$18, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
         <v/>
       </c>
       <c r="N23" t="str" cm="1">
-        <f t="array" ref="N23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$18, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="8"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+        <f t="array" ref="N23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A24" s="8">
+        <v>22</v>
+      </c>
+      <c r="B24" t="e" cm="1">
+        <f t="array" ref="B24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C24" t="e" cm="1">
+        <f t="array" ref="C24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D24" t="e" cm="1">
+        <f t="array" ref="D24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E24" t="e" cm="1">
+        <f t="array" ref="E24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F24" t="e" cm="1">
+        <f t="array" ref="F24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G24" t="e" cm="1">
+        <f t="array" ref="G24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H24" t="e" cm="1">
+        <f t="array" ref="H24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I24" t="e" cm="1">
+        <f t="array" ref="I24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J24" t="e" cm="1">
+        <f t="array" ref="J24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K24" t="e" cm="1">
+        <f t="array" ref="K24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L24" t="str" cm="1">
+        <f t="array" ref="L24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M24" t="str" cm="1">
+        <f t="array" ref="M24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="N24" t="str" cm="1">
+        <f t="array" ref="N24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="8"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="8"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="8"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="8"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="8"/>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A30" s="8"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31" s="8"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
@@ -2782,6 +2899,9 @@
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" s="8"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" s="8"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1:Q1 B2:K1048576">

</xml_diff>

<commit_message>
LC -> LU conversion: - Updated with more suggested exceptions and scenarios (i.e. tree crops and temporary flooded veg)
</commit_message>
<xml_diff>
--- a/src/LULUCF/scripts/postprocessing/conversion_LUC_scenarios.xlsx
+++ b/src/LULUCF/scripts/postprocessing/conversion_LUC_scenarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\git\AFOLU_GHG_flux_model\src\LULUCF\scripts\postprocessing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9837866C-F0CA-4217-9EAB-030630691D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47BB6BE-D6BB-46CE-A074-6A6D86CA4E23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="62">
   <si>
     <t>Driver</t>
   </si>
@@ -135,9 +135,6 @@
     <t>forest wet</t>
   </si>
   <si>
-    <t>sdpt</t>
-  </si>
-  <si>
     <t>logging_concession</t>
   </si>
   <si>
@@ -213,9 +210,6 @@
     <t>Forest to cropland in 2022</t>
   </si>
   <si>
-    <t>or should this be cropland remaining cropland</t>
-  </si>
-  <si>
     <t>*</t>
   </si>
   <si>
@@ -223,6 +217,36 @@
   </si>
   <si>
     <t xml:space="preserve">Forest to cropland in 2017 </t>
+  </si>
+  <si>
+    <t>or Forest remaining Forest since driver is not shifting cultivation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cropland to forest then forest to cropland </t>
+  </si>
+  <si>
+    <t>sdpt_type</t>
+  </si>
+  <si>
+    <t>sdpt_name</t>
+  </si>
+  <si>
+    <t>establishment_year</t>
+  </si>
+  <si>
+    <t>Forest land to crop land in 2020</t>
+  </si>
+  <si>
+    <t>or Forest land to cropland in 2020?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should this be forest remaining forest? </t>
+  </si>
+  <si>
+    <t>Forest to grassland in 2018</t>
+  </si>
+  <si>
+    <t>Forest to grass to forest in 2017 right now</t>
   </si>
 </sst>
 </file>
@@ -307,7 +331,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill>
@@ -333,6 +357,13 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -621,61 +652,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="8"/>
     <col min="12" max="12" width="9.21875" customWidth="1"/>
-    <col min="13" max="13" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>21</v>
       </c>
       <c r="M1" t="s">
+        <v>54</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="O1" t="s">
+        <v>56</v>
+      </c>
+      <c r="P1" t="s">
         <v>24</v>
       </c>
-      <c r="N1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -709,11 +748,11 @@
       <c r="K2">
         <v>1</v>
       </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -751,7 +790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -786,7 +825,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -821,7 +860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -856,7 +895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>6</v>
       </c>
@@ -894,7 +933,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -932,7 +971,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -967,7 +1006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>9</v>
       </c>
@@ -1003,7 +1042,7 @@
       </c>
       <c r="L10" s="6"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>10</v>
       </c>
@@ -1039,7 +1078,7 @@
       </c>
       <c r="L11" s="6"/>
     </row>
-    <row r="12" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>11</v>
       </c>
@@ -1075,7 +1114,7 @@
       </c>
       <c r="L12" s="6"/>
     </row>
-    <row r="13" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>12</v>
       </c>
@@ -1111,7 +1150,7 @@
       </c>
       <c r="L13" s="7"/>
     </row>
-    <row r="14" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>13</v>
       </c>
@@ -1149,7 +1188,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>14</v>
       </c>
@@ -1187,7 +1226,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>15</v>
       </c>
@@ -1225,7 +1264,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>16</v>
       </c>
@@ -1263,7 +1302,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>17</v>
       </c>
@@ -1299,7 +1338,7 @@
       </c>
       <c r="L18" s="7"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>18</v>
       </c>
@@ -1335,6 +1374,214 @@
       </c>
       <c r="L19" s="7">
         <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A20" s="8">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1">
+        <v>3</v>
+      </c>
+      <c r="C20" s="1">
+        <v>3</v>
+      </c>
+      <c r="D20" s="1">
+        <v>3</v>
+      </c>
+      <c r="E20" s="1">
+        <v>3</v>
+      </c>
+      <c r="F20" s="1">
+        <v>3</v>
+      </c>
+      <c r="G20" s="1">
+        <v>1</v>
+      </c>
+      <c r="H20" s="1">
+        <v>1</v>
+      </c>
+      <c r="I20" s="1">
+        <v>1</v>
+      </c>
+      <c r="J20" s="1">
+        <v>1</v>
+      </c>
+      <c r="K20" s="1">
+        <v>1</v>
+      </c>
+      <c r="L20" s="7">
+        <v>3</v>
+      </c>
+      <c r="M20">
+        <v>2</v>
+      </c>
+      <c r="N20">
+        <v>1</v>
+      </c>
+      <c r="O20">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A21" s="8">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1">
+        <v>3</v>
+      </c>
+      <c r="C21" s="1">
+        <v>3</v>
+      </c>
+      <c r="D21" s="1">
+        <v>3</v>
+      </c>
+      <c r="E21" s="1">
+        <v>3</v>
+      </c>
+      <c r="F21" s="1">
+        <v>3</v>
+      </c>
+      <c r="G21" s="1">
+        <v>1</v>
+      </c>
+      <c r="H21" s="1">
+        <v>1</v>
+      </c>
+      <c r="I21" s="1">
+        <v>1</v>
+      </c>
+      <c r="J21" s="1">
+        <v>1</v>
+      </c>
+      <c r="K21" s="1">
+        <v>1</v>
+      </c>
+      <c r="L21" s="7">
+        <v>3</v>
+      </c>
+      <c r="M21">
+        <v>2</v>
+      </c>
+      <c r="N21">
+        <v>1</v>
+      </c>
+      <c r="O21">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A22" s="8">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>3</v>
+      </c>
+      <c r="C22" s="1">
+        <v>3</v>
+      </c>
+      <c r="D22" s="1">
+        <v>3</v>
+      </c>
+      <c r="E22" s="1">
+        <v>3</v>
+      </c>
+      <c r="F22" s="1">
+        <v>3</v>
+      </c>
+      <c r="G22" s="1">
+        <v>1</v>
+      </c>
+      <c r="H22" s="1">
+        <v>1</v>
+      </c>
+      <c r="I22" s="1">
+        <v>1</v>
+      </c>
+      <c r="J22" s="1">
+        <v>1</v>
+      </c>
+      <c r="K22" s="1">
+        <v>1</v>
+      </c>
+      <c r="L22" s="7">
+        <v>3</v>
+      </c>
+      <c r="M22" s="1">
+        <v>2</v>
+      </c>
+      <c r="N22" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23" s="8">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1">
+        <v>3</v>
+      </c>
+      <c r="C23" s="1">
+        <v>1</v>
+      </c>
+      <c r="D23" s="1">
+        <v>4</v>
+      </c>
+      <c r="E23" s="1">
+        <v>1</v>
+      </c>
+      <c r="F23" s="1">
+        <v>3</v>
+      </c>
+      <c r="G23" s="1">
+        <v>1</v>
+      </c>
+      <c r="H23" s="1">
+        <v>4</v>
+      </c>
+      <c r="I23" s="1">
+        <v>1</v>
+      </c>
+      <c r="J23" s="1">
+        <v>3</v>
+      </c>
+      <c r="K23" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A24" s="8">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1">
+        <v>3</v>
+      </c>
+      <c r="C24" s="1">
+        <v>3</v>
+      </c>
+      <c r="D24" s="1">
+        <v>3</v>
+      </c>
+      <c r="E24" s="1">
+        <v>4</v>
+      </c>
+      <c r="F24" s="1">
+        <v>1</v>
+      </c>
+      <c r="G24" s="1">
+        <v>4</v>
+      </c>
+      <c r="H24" s="1">
+        <v>1</v>
+      </c>
+      <c r="I24" s="1">
+        <v>4</v>
+      </c>
+      <c r="J24" s="1">
+        <v>1</v>
+      </c>
+      <c r="K24" s="1">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1344,14 +1591,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FD5E73A-BF21-4771-A2AF-1B9A394A8B1D}">
-  <dimension ref="A1:T66"/>
+  <dimension ref="A1:W66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="12" max="12" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="31.109375" customWidth="1"/>
+    <col min="22" max="22" width="31.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>2</v>
       </c>
@@ -1392,1413 +1639,1637 @@
         <v>14</v>
       </c>
       <c r="O1">
+        <v>15</v>
+      </c>
+      <c r="P1">
+        <v>16</v>
+      </c>
+      <c r="Q1">
+        <v>17</v>
+      </c>
+      <c r="R1">
         <v>18</v>
       </c>
-      <c r="P1">
+      <c r="S1">
         <v>19</v>
       </c>
-      <c r="Q1">
+      <c r="T1">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="M2" t="s">
+        <v>54</v>
+      </c>
+      <c r="N2" t="s">
+        <v>55</v>
+      </c>
+      <c r="O2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P2" t="s">
         <v>24</v>
       </c>
-      <c r="N2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="T2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>1</v>
       </c>
       <c r="B3" t="str" cm="1">
-        <f t="array" ref="B3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="C3" t="str" cm="1">
-        <f t="array" ref="C3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D3" t="str" cm="1">
-        <f t="array" ref="D3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E3" t="str" cm="1">
-        <f t="array" ref="E3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F3" t="str" cm="1">
-        <f t="array" ref="F3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G3" t="str" cm="1">
-        <f t="array" ref="G3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H3" t="str" cm="1">
-        <f t="array" ref="H3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I3" t="str" cm="1">
-        <f t="array" ref="I3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J3" t="str" cm="1">
-        <f t="array" ref="J3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="K3" t="str" cm="1">
-        <f t="array" ref="K3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K3">_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L3" t="str" cm="1">
-        <f t="array" ref="L3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M3" t="str" cm="1">
-        <f t="array" ref="M3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N3" t="str" cm="1">
-        <f t="array" ref="N3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
+        <f t="array" ref="N3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="P3" t="str" cm="1">
+        <f t="array" ref="P3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$P$100, P$1, 0), 1, "yes"), "")</f>
         <v>yes</v>
       </c>
-      <c r="Q3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="Q3" t="str" cm="1">
+        <f t="array" ref="Q3">IFERROR(_xlfn.SWITCH(VLOOKUP($A3, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>2</v>
       </c>
       <c r="B4" t="str" cm="1">
-        <f t="array" ref="B4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="C4" t="str" cm="1">
-        <f t="array" ref="C4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D4" t="str" cm="1">
-        <f t="array" ref="D4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E4" t="str" cm="1">
-        <f t="array" ref="E4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F4" t="str" cm="1">
-        <f t="array" ref="F4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G4" t="str" cm="1">
-        <f t="array" ref="G4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H4" t="str" cm="1">
-        <f t="array" ref="H4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I4" t="str" cm="1">
-        <f t="array" ref="I4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J4" t="str" cm="1">
-        <f t="array" ref="J4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="K4" t="str" cm="1">
-        <f t="array" ref="K4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K4">_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L4" t="str" cm="1">
-        <f t="array" ref="L4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M4" t="str" cm="1">
-        <f t="array" ref="M4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v>oil palm</v>
+        <f t="array" ref="M4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
+        <v>planted forest</v>
       </c>
       <c r="N4" t="str" cm="1">
-        <f t="array" ref="N4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q4" t="s">
+        <f t="array" ref="N4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q4" t="str" cm="1">
+        <f t="array" ref="Q4">IFERROR(_xlfn.SWITCH(VLOOKUP($A4, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A5" s="8">
+        <v>3</v>
+      </c>
+      <c r="B5" t="str" cm="1">
+        <f t="array" ref="B5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="C5" t="str" cm="1">
+        <f t="array" ref="C5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D5" t="str" cm="1">
+        <f t="array" ref="D5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="E5" t="str" cm="1">
+        <f t="array" ref="E5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="F5" t="str" cm="1">
+        <f t="array" ref="F5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="G5" t="str" cm="1">
+        <f t="array" ref="G5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="H5" t="str" cm="1">
+        <f t="array" ref="H5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="I5" t="str" cm="1">
+        <f t="array" ref="I5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="J5" t="str" cm="1">
+        <f t="array" ref="J5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="K5" t="str" cm="1">
+        <f t="array" ref="K5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="L5" t="str" cm="1">
+        <f t="array" ref="L5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M5" t="str" cm="1">
+        <f t="array" ref="M5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
+        <v/>
+      </c>
+      <c r="N5" t="str" cm="1">
+        <f t="array" ref="N5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q5" t="str" cm="1">
+        <f t="array" ref="Q5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A5" s="8">
-        <v>3</v>
-      </c>
-      <c r="B5" t="str" cm="1">
-        <f t="array" ref="B5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="C5" t="str" cm="1">
-        <f t="array" ref="C5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="D5" t="str" cm="1">
-        <f t="array" ref="D5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="E5" t="str" cm="1">
-        <f t="array" ref="E5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="F5" t="str" cm="1">
-        <f t="array" ref="F5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="G5" t="str" cm="1">
-        <f t="array" ref="G5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="H5" t="str" cm="1">
-        <f t="array" ref="H5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="I5" t="str" cm="1">
-        <f t="array" ref="I5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="J5" t="str" cm="1">
-        <f t="array" ref="J5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="K5" t="str" cm="1">
-        <f t="array" ref="K5">_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="L5" t="str" cm="1">
-        <f t="array" ref="L5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="M5" t="str" cm="1">
-        <f t="array" ref="M5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="N5" t="str" cm="1">
-        <f t="array" ref="N5">IFERROR(_xlfn.SWITCH(VLOOKUP($A5, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>4</v>
       </c>
       <c r="B6" t="str" cm="1">
-        <f t="array" ref="B6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C6" t="str" cm="1">
-        <f t="array" ref="C6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D6" t="str" cm="1">
-        <f t="array" ref="D6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E6" t="str" cm="1">
-        <f t="array" ref="E6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F6" t="str" cm="1">
-        <f t="array" ref="F6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G6" t="str" cm="1">
-        <f t="array" ref="G6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H6" t="str" cm="1">
-        <f t="array" ref="H6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I6" t="str" cm="1">
-        <f t="array" ref="I6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J6" t="str" cm="1">
-        <f t="array" ref="J6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K6" t="str" cm="1">
-        <f t="array" ref="K6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K6">_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L6" t="str" cm="1">
-        <f t="array" ref="L6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M6" t="str" cm="1">
-        <f t="array" ref="M6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N6" t="str" cm="1">
-        <f t="array" ref="N6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q6" t="str" cm="1">
+        <f t="array" ref="Q6">IFERROR(_xlfn.SWITCH(VLOOKUP($A6, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>5</v>
       </c>
       <c r="B7" t="str" cm="1">
-        <f t="array" ref="B7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C7" t="str" cm="1">
-        <f t="array" ref="C7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D7" t="str" cm="1">
-        <f t="array" ref="D7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E7" t="str" cm="1">
-        <f t="array" ref="E7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F7" t="str" cm="1">
-        <f t="array" ref="F7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G7" t="str" cm="1">
-        <f t="array" ref="G7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H7" t="str" cm="1">
-        <f t="array" ref="H7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I7" t="str" cm="1">
-        <f t="array" ref="I7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J7" t="str" cm="1">
-        <f t="array" ref="J7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K7" t="str" cm="1">
-        <f t="array" ref="K7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K7">_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L7" t="str" cm="1">
-        <f t="array" ref="L7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M7" t="str" cm="1">
-        <f t="array" ref="M7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N7" t="str" cm="1">
-        <f t="array" ref="N7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q7" t="str" cm="1">
+        <f t="array" ref="Q7">IFERROR(_xlfn.SWITCH(VLOOKUP($A7, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>6</v>
       </c>
       <c r="B8" t="str" cm="1">
-        <f t="array" ref="B8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="C8" t="str" cm="1">
-        <f t="array" ref="C8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="D8" t="str" cm="1">
-        <f t="array" ref="D8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E8" t="str" cm="1">
-        <f t="array" ref="E8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F8" t="str" cm="1">
-        <f t="array" ref="F8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G8" t="str" cm="1">
-        <f t="array" ref="G8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H8" t="str" cm="1">
-        <f t="array" ref="H8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I8" t="str" cm="1">
-        <f t="array" ref="I8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="J8" t="str" cm="1">
-        <f t="array" ref="J8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K8" t="str" cm="1">
-        <f t="array" ref="K8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K8">_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="L8" t="str" cm="1">
-        <f t="array" ref="L8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Logging</v>
       </c>
       <c r="M8" t="str" cm="1">
-        <f t="array" ref="M8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N8" t="str" cm="1">
-        <f t="array" ref="N8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q8" t="s">
+        <f t="array" ref="N8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q8" t="str" cm="1">
+        <f t="array" ref="Q8">IFERROR(_xlfn.SWITCH(VLOOKUP($A8, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A9" s="8">
+        <v>7</v>
+      </c>
+      <c r="B9" t="str" cm="1">
+        <f t="array" ref="B9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C9" t="str" cm="1">
+        <f t="array" ref="C9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D9" t="str" cm="1">
+        <f t="array" ref="D9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="E9" t="str" cm="1">
+        <f t="array" ref="E9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="F9" t="str" cm="1">
+        <f t="array" ref="F9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="G9" t="str" cm="1">
+        <f t="array" ref="G9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="H9" t="str" cm="1">
+        <f t="array" ref="H9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="I9" t="str" cm="1">
+        <f t="array" ref="I9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="J9" t="str" cm="1">
+        <f t="array" ref="J9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="K9" t="str" cm="1">
+        <f t="array" ref="K9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="L9" t="str" cm="1">
+        <f t="array" ref="L9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Logging</v>
+      </c>
+      <c r="M9" t="str" cm="1">
+        <f t="array" ref="M9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
+        <v/>
+      </c>
+      <c r="N9" t="str" cm="1">
+        <f t="array" ref="N9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q9" t="str" cm="1">
+        <f t="array" ref="Q9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A9" s="8">
-        <v>7</v>
-      </c>
-      <c r="B9" t="str" cm="1">
-        <f t="array" ref="B9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="C9" t="str" cm="1">
-        <f t="array" ref="C9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="D9" t="str" cm="1">
-        <f t="array" ref="D9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>tall veg</v>
-      </c>
-      <c r="E9" t="str" cm="1">
-        <f t="array" ref="E9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="F9" t="str" cm="1">
-        <f t="array" ref="F9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="G9" t="str" cm="1">
-        <f t="array" ref="G9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="H9" t="str" cm="1">
-        <f t="array" ref="H9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="I9" t="str" cm="1">
-        <f t="array" ref="I9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="J9" t="str" cm="1">
-        <f t="array" ref="J9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="K9" t="str" cm="1">
-        <f t="array" ref="K9">_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="L9" t="str" cm="1">
-        <f t="array" ref="L9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v>Logging</v>
-      </c>
-      <c r="M9" t="str" cm="1">
-        <f t="array" ref="M9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="N9" t="str" cm="1">
-        <f t="array" ref="N9">IFERROR(_xlfn.SWITCH(VLOOKUP($A9, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>8</v>
       </c>
       <c r="B10" t="str" cm="1">
-        <f t="array" ref="B10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C10" t="str" cm="1">
-        <f t="array" ref="C10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D10" t="str" cm="1">
-        <f t="array" ref="D10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="E10" t="str" cm="1">
-        <f t="array" ref="E10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F10" t="str" cm="1">
-        <f t="array" ref="F10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="G10" t="str" cm="1">
-        <f t="array" ref="G10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="H10" t="str" cm="1">
-        <f t="array" ref="H10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="I10" t="str" cm="1">
-        <f t="array" ref="I10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J10" t="str" cm="1">
-        <f t="array" ref="J10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="K10" t="str" cm="1">
-        <f t="array" ref="K10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K10">_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L10" t="str" cm="1">
-        <f t="array" ref="L10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M10" t="str" cm="1">
-        <f t="array" ref="M10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N10" t="str" cm="1">
-        <f t="array" ref="N10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q10" t="str" cm="1">
+        <f t="array" ref="Q10">IFERROR(_xlfn.SWITCH(VLOOKUP($A10, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>9</v>
       </c>
       <c r="B11" t="str" cm="1">
-        <f t="array" ref="B11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C11" t="str" cm="1">
-        <f t="array" ref="C11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D11" t="str" cm="1">
-        <f t="array" ref="D11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E11" t="str" cm="1">
-        <f t="array" ref="E11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F11" t="str" cm="1">
-        <f t="array" ref="F11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G11" t="str" cm="1">
-        <f t="array" ref="G11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H11" t="str" cm="1">
-        <f t="array" ref="H11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I11" t="str" cm="1">
-        <f t="array" ref="I11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="J11" t="str" cm="1">
-        <f t="array" ref="J11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K11" t="str" cm="1">
-        <f t="array" ref="K11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K11">_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="L11" t="str" cm="1">
-        <f t="array" ref="L11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M11" t="str" cm="1">
-        <f t="array" ref="M11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N11" t="str" cm="1">
-        <f t="array" ref="N11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q11" t="s">
+        <f t="array" ref="N11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q11" t="str" cm="1">
+        <f t="array" ref="Q11">IFERROR(_xlfn.SWITCH(VLOOKUP($A11, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A12" s="8">
+        <v>10</v>
+      </c>
+      <c r="B12" t="str" cm="1">
+        <f t="array" ref="B12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="C12" t="str" cm="1">
+        <f t="array" ref="C12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="D12" t="str" cm="1">
+        <f t="array" ref="D12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="E12" t="str" cm="1">
+        <f t="array" ref="E12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="F12" t="str" cm="1">
+        <f t="array" ref="F12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="G12" t="str" cm="1">
+        <f t="array" ref="G12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="H12" t="str" cm="1">
+        <f t="array" ref="H12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="I12" t="str" cm="1">
+        <f t="array" ref="I12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="J12" t="str" cm="1">
+        <f t="array" ref="J12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="K12" t="str" cm="1">
+        <f t="array" ref="K12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="L12" t="str" cm="1">
+        <f t="array" ref="L12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M12" t="str" cm="1">
+        <f t="array" ref="M12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
+        <v/>
+      </c>
+      <c r="N12" t="str" cm="1">
+        <f t="array" ref="N12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q12" t="str" cm="1">
+        <f t="array" ref="Q12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T12" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A12" s="8">
-        <v>10</v>
-      </c>
-      <c r="B12" t="str" cm="1">
-        <f t="array" ref="B12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="C12" t="str" cm="1">
-        <f t="array" ref="C12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="D12" t="str" cm="1">
-        <f t="array" ref="D12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="E12" t="str" cm="1">
-        <f t="array" ref="E12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="F12" t="str" cm="1">
-        <f t="array" ref="F12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="G12" t="str" cm="1">
-        <f t="array" ref="G12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="H12" t="str" cm="1">
-        <f t="array" ref="H12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="I12" t="str" cm="1">
-        <f t="array" ref="I12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="J12" t="str" cm="1">
-        <f t="array" ref="J12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="K12" t="str" cm="1">
-        <f t="array" ref="K12">_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>short veg</v>
-      </c>
-      <c r="L12" t="str" cm="1">
-        <f t="array" ref="L12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
-      </c>
-      <c r="M12" t="str" cm="1">
-        <f t="array" ref="M12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
-      </c>
-      <c r="N12" t="str" cm="1">
-        <f t="array" ref="N12">IFERROR(_xlfn.SWITCH(VLOOKUP($A12, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q12" t="s">
-        <v>39</v>
-      </c>
-      <c r="T12" s="9"/>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="W12" s="9"/>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>11</v>
       </c>
       <c r="B13" t="str" cm="1">
-        <f t="array" ref="B13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="C13" t="str" cm="1">
-        <f t="array" ref="C13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="D13" t="str" cm="1">
-        <f t="array" ref="D13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="E13" t="str" cm="1">
-        <f t="array" ref="E13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="F13" t="str" cm="1">
-        <f t="array" ref="F13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="G13" t="str" cm="1">
-        <f t="array" ref="G13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="H13" t="str" cm="1">
-        <f t="array" ref="H13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="I13" t="str" cm="1">
-        <f t="array" ref="I13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J13" t="str" cm="1">
-        <f t="array" ref="J13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K13" t="str" cm="1">
-        <f t="array" ref="K13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K13">_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L13" t="str" cm="1">
-        <f t="array" ref="L13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M13" t="str" cm="1">
-        <f t="array" ref="M13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N13" t="str" cm="1">
-        <f t="array" ref="N13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q13" t="s">
-        <v>40</v>
-      </c>
-      <c r="T13" s="9"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q13" t="str" cm="1">
+        <f t="array" ref="Q13">IFERROR(_xlfn.SWITCH(VLOOKUP($A13, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T13" t="s">
+        <v>39</v>
+      </c>
+      <c r="W13" s="9"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>12</v>
       </c>
       <c r="B14" t="str" cm="1">
-        <f t="array" ref="B14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C14" t="str" cm="1">
-        <f t="array" ref="C14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D14" t="str" cm="1">
-        <f t="array" ref="D14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E14" t="str" cm="1">
-        <f t="array" ref="E14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F14" t="str" cm="1">
-        <f t="array" ref="F14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G14" t="str" cm="1">
-        <f t="array" ref="G14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H14" t="str" cm="1">
-        <f t="array" ref="H14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I14" t="str" cm="1">
-        <f t="array" ref="I14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J14" t="str" cm="1">
-        <f t="array" ref="J14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K14" t="str" cm="1">
-        <f t="array" ref="K14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K14">_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L14" t="str" cm="1">
-        <f t="array" ref="L14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M14" t="str" cm="1">
-        <f t="array" ref="M14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N14" t="str" cm="1">
-        <f t="array" ref="N14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q14" t="s">
+        <f t="array" ref="N14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q14" t="str" cm="1">
+        <f t="array" ref="Q14">IFERROR(_xlfn.SWITCH(VLOOKUP($A14, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="S14" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="T14" t="s">
+        <v>48</v>
+      </c>
+      <c r="W14" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>13</v>
       </c>
       <c r="B15" t="str" cm="1">
-        <f t="array" ref="B15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C15" t="str" cm="1">
-        <f t="array" ref="C15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D15" t="str" cm="1">
-        <f t="array" ref="D15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E15" t="str" cm="1">
-        <f t="array" ref="E15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F15" t="str" cm="1">
-        <f t="array" ref="F15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G15" t="str" cm="1">
-        <f t="array" ref="G15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H15" t="str" cm="1">
-        <f t="array" ref="H15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I15" t="str" cm="1">
-        <f t="array" ref="I15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J15" t="str" cm="1">
-        <f t="array" ref="J15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K15" t="str" cm="1">
-        <f t="array" ref="K15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K15">_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L15" t="str" cm="1">
-        <f t="array" ref="L15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Shifting cultivation</v>
       </c>
       <c r="M15" t="str" cm="1">
-        <f t="array" ref="M15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N15" t="str" cm="1">
-        <f t="array" ref="N15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q15" t="s">
+        <f t="array" ref="N15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q15" t="str" cm="1">
+        <f t="array" ref="Q15">IFERROR(_xlfn.SWITCH(VLOOKUP($A15, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="S15" t="s">
         <v>49</v>
       </c>
       <c r="T15" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+      <c r="W15" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>14</v>
       </c>
       <c r="B16" t="str" cm="1">
-        <f t="array" ref="B16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C16" t="str" cm="1">
-        <f t="array" ref="C16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D16" t="str" cm="1">
-        <f t="array" ref="D16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="E16" t="str" cm="1">
-        <f t="array" ref="E16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="F16" t="str" cm="1">
-        <f t="array" ref="F16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G16" t="str" cm="1">
-        <f t="array" ref="G16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H16" t="str" cm="1">
-        <f t="array" ref="H16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I16" t="str" cm="1">
-        <f t="array" ref="I16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J16" t="str" cm="1">
-        <f t="array" ref="J16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K16" t="str" cm="1">
-        <f t="array" ref="K16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K16">_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L16" t="str" cm="1">
-        <f t="array" ref="L16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Shifting cultivation</v>
       </c>
       <c r="M16" t="str" cm="1">
-        <f t="array" ref="M16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N16" t="str" cm="1">
-        <f t="array" ref="N16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q16" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q16" t="str" cm="1">
+        <f t="array" ref="Q16">IFERROR(_xlfn.SWITCH(VLOOKUP($A16, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="S16" t="s">
+        <v>49</v>
+      </c>
+      <c r="T16" t="s">
+        <v>51</v>
+      </c>
+      <c r="W16" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>15</v>
       </c>
       <c r="B17" t="str" cm="1">
-        <f t="array" ref="B17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C17" t="str" cm="1">
-        <f t="array" ref="C17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D17" t="str" cm="1">
-        <f t="array" ref="D17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E17" t="str" cm="1">
-        <f t="array" ref="E17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="F17" t="str" cm="1">
-        <f t="array" ref="F17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G17" t="str" cm="1">
-        <f t="array" ref="G17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H17" t="str" cm="1">
-        <f t="array" ref="H17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I17" t="str" cm="1">
-        <f t="array" ref="I17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J17" t="str" cm="1">
-        <f t="array" ref="J17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K17" t="str" cm="1">
-        <f t="array" ref="K17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K17">_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L17" t="str" cm="1">
-        <f t="array" ref="L17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Shifting cultivation</v>
       </c>
       <c r="M17" t="str" cm="1">
-        <f t="array" ref="M17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N17" t="str" cm="1">
-        <f t="array" ref="N17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q17" t="s">
-        <v>52</v>
-      </c>
-      <c r="T17" s="9" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q17" t="str" cm="1">
+        <f t="array" ref="Q17">IFERROR(_xlfn.SWITCH(VLOOKUP($A17, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="S17" t="s">
+        <v>49</v>
+      </c>
+      <c r="T17" t="s">
+        <v>50</v>
+      </c>
+      <c r="W17" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>16</v>
       </c>
       <c r="B18" t="str" cm="1">
-        <f t="array" ref="B18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C18" t="str" cm="1">
-        <f t="array" ref="C18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D18" t="str" cm="1">
-        <f t="array" ref="D18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E18" t="str" cm="1">
-        <f t="array" ref="E18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="F18" t="str" cm="1">
-        <f t="array" ref="F18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G18" t="str" cm="1">
-        <f t="array" ref="G18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H18" t="str" cm="1">
-        <f t="array" ref="H18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I18" t="str" cm="1">
-        <f t="array" ref="I18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="J18" t="str" cm="1">
-        <f t="array" ref="J18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="K18" t="str" cm="1">
-        <f t="array" ref="K18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K18">_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>short veg</v>
       </c>
       <c r="L18" t="str" cm="1">
-        <f t="array" ref="L18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Shifting cultivation</v>
       </c>
       <c r="M18" t="str" cm="1">
-        <f t="array" ref="M18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N18" t="str" cm="1">
-        <f t="array" ref="N18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="P18" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>52</v>
-      </c>
-      <c r="T18" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q18" t="str" cm="1">
+        <f t="array" ref="Q18">IFERROR(_xlfn.SWITCH(VLOOKUP($A18, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="S18" t="s">
+        <v>49</v>
+      </c>
+      <c r="T18" t="s">
+        <v>50</v>
+      </c>
+      <c r="W18" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>17</v>
       </c>
       <c r="B19" t="str" cm="1">
-        <f t="array" ref="B19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="C19" t="str" cm="1">
-        <f t="array" ref="C19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D19" t="str" cm="1">
-        <f t="array" ref="D19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E19" t="str" cm="1">
-        <f t="array" ref="E19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="F19" t="str" cm="1">
-        <f t="array" ref="F19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="G19" t="str" cm="1">
-        <f t="array" ref="G19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="H19" t="str" cm="1">
-        <f t="array" ref="H19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="I19" t="str" cm="1">
-        <f t="array" ref="I19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="J19" t="str" cm="1">
-        <f t="array" ref="J19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="K19" t="str" cm="1">
-        <f t="array" ref="K19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K19">_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>cropland</v>
       </c>
       <c r="L19" t="str" cm="1">
-        <f t="array" ref="L19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M19" t="str" cm="1">
-        <f t="array" ref="M19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N19" t="str" cm="1">
-        <f t="array" ref="N19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="Q19" t="s">
-        <v>40</v>
-      </c>
-      <c r="T19" s="9"/>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q19" t="str" cm="1">
+        <f t="array" ref="Q19">IFERROR(_xlfn.SWITCH(VLOOKUP($A19, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="S19" t="s">
+        <v>49</v>
+      </c>
+      <c r="T19" t="s">
+        <v>53</v>
+      </c>
+      <c r="W19" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>18</v>
       </c>
       <c r="B20" t="str" cm="1">
-        <f t="array" ref="B20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="B20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="C20" t="str" cm="1">
-        <f t="array" ref="C20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="C20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="D20" t="str" cm="1">
-        <f t="array" ref="D20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="D20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="E20" t="str" cm="1">
-        <f t="array" ref="E20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="E20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="F20" t="str" cm="1">
-        <f t="array" ref="F20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="F20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="G20" t="str" cm="1">
-        <f t="array" ref="G20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="G20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="H20" t="str" cm="1">
-        <f t="array" ref="H20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="H20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="I20" t="str" cm="1">
-        <f t="array" ref="I20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="I20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="J20" t="str" cm="1">
-        <f t="array" ref="J20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="J20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="K20" t="str" cm="1">
-        <f t="array" ref="K20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <f t="array" ref="K20">_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
         <v>tall veg</v>
       </c>
       <c r="L20" t="str" cm="1">
-        <f t="array" ref="L20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v>Shifting cultivation</v>
       </c>
       <c r="M20" t="str" cm="1">
-        <f t="array" ref="M20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N20" t="str" cm="1">
-        <f t="array" ref="N20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-      <c r="P20" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q20" t="s">
+        <f t="array" ref="N20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q20" t="str" cm="1">
+        <f t="array" ref="Q20">IFERROR(_xlfn.SWITCH(VLOOKUP($A20, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="S20" t="s">
+        <v>49</v>
+      </c>
+      <c r="T20" t="s">
+        <v>40</v>
+      </c>
+      <c r="W20" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="T20" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
         <v>19</v>
       </c>
-      <c r="B21" t="e" cm="1">
-        <f t="array" ref="B21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="C21" t="e" cm="1">
-        <f t="array" ref="C21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D21" t="e" cm="1">
-        <f t="array" ref="D21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E21" t="e" cm="1">
-        <f t="array" ref="E21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F21" t="e" cm="1">
-        <f t="array" ref="F21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G21" t="e" cm="1">
-        <f t="array" ref="G21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H21" t="e" cm="1">
-        <f t="array" ref="H21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="I21" t="e" cm="1">
-        <f t="array" ref="I21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="J21" t="e" cm="1">
-        <f t="array" ref="J21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K21" t="e" cm="1">
-        <f t="array" ref="K21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
+      <c r="B21" t="str" cm="1">
+        <f t="array" ref="B21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C21" t="str" cm="1">
+        <f t="array" ref="C21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D21" t="str" cm="1">
+        <f t="array" ref="D21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="E21" t="str" cm="1">
+        <f t="array" ref="E21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="F21" t="str" cm="1">
+        <f t="array" ref="F21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="G21" t="str" cm="1">
+        <f t="array" ref="G21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="H21" t="str" cm="1">
+        <f t="array" ref="H21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="I21" t="str" cm="1">
+        <f t="array" ref="I21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="J21" t="str" cm="1">
+        <f t="array" ref="J21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="K21" t="str" cm="1">
+        <f t="array" ref="K21">_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L21" t="str" cm="1">
-        <f t="array" ref="L21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
+        <f t="array" ref="L21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M21" t="str" cm="1">
-        <f t="array" ref="M21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
+        <f t="array" ref="M21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
+        <v>tree crop</v>
       </c>
       <c r="N21" t="str" cm="1">
-        <f t="array" ref="N21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v>oil palm</v>
+      </c>
+      <c r="O21">
+        <f>IFERROR(VLOOKUP($A21, scenarios!$A$2:$P$100, O$1, 0), "")</f>
+        <v>2000</v>
+      </c>
+      <c r="Q21" t="str" cm="1">
+        <f t="array" ref="Q21">IFERROR(_xlfn.SWITCH(VLOOKUP($A21, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>20</v>
       </c>
-      <c r="B22" t="e" cm="1">
-        <f t="array" ref="B22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="C22" t="e" cm="1">
-        <f t="array" ref="C22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D22" t="e" cm="1">
-        <f t="array" ref="D22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E22" t="e" cm="1">
-        <f t="array" ref="E22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F22" t="e" cm="1">
-        <f t="array" ref="F22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G22" t="e" cm="1">
-        <f t="array" ref="G22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H22" t="e" cm="1">
-        <f t="array" ref="H22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="I22" t="e" cm="1">
-        <f t="array" ref="I22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="J22" t="e" cm="1">
-        <f t="array" ref="J22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K22" t="e" cm="1">
-        <f t="array" ref="K22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
+      <c r="B22" t="str" cm="1">
+        <f t="array" ref="B22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C22" t="str" cm="1">
+        <f t="array" ref="C22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D22" t="str" cm="1">
+        <f t="array" ref="D22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="E22" t="str" cm="1">
+        <f t="array" ref="E22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="F22" t="str" cm="1">
+        <f t="array" ref="F22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="G22" t="str" cm="1">
+        <f t="array" ref="G22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="H22" t="str" cm="1">
+        <f t="array" ref="H22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="I22" t="str" cm="1">
+        <f t="array" ref="I22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="J22" t="str" cm="1">
+        <f t="array" ref="J22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="K22" t="str" cm="1">
+        <f t="array" ref="K22">_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L22" t="str" cm="1">
-        <f t="array" ref="L22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
+        <f t="array" ref="L22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M22" t="str" cm="1">
-        <f t="array" ref="M22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
+        <f t="array" ref="M22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
+        <v>tree crop</v>
       </c>
       <c r="N22" t="str" cm="1">
-        <f t="array" ref="N22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v>oil palm</v>
+      </c>
+      <c r="O22">
+        <f>IFERROR(VLOOKUP($A22, scenarios!$A$2:$P$100, O$1, 0), "")</f>
+        <v>2020</v>
+      </c>
+      <c r="Q22" t="str" cm="1">
+        <f t="array" ref="Q22">IFERROR(_xlfn.SWITCH(VLOOKUP($A22, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
         <v>21</v>
       </c>
-      <c r="B23" t="e" cm="1">
-        <f t="array" ref="B23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="C23" t="e" cm="1">
-        <f t="array" ref="C23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D23" t="e" cm="1">
-        <f t="array" ref="D23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E23" t="e" cm="1">
-        <f t="array" ref="E23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F23" t="e" cm="1">
-        <f t="array" ref="F23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G23" t="e" cm="1">
-        <f t="array" ref="G23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H23" t="e" cm="1">
-        <f t="array" ref="H23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="I23" t="e" cm="1">
-        <f t="array" ref="I23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="J23" t="e" cm="1">
-        <f t="array" ref="J23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K23" t="e" cm="1">
-        <f t="array" ref="K23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
+      <c r="B23" t="str" cm="1">
+        <f t="array" ref="B23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C23" t="str" cm="1">
+        <f t="array" ref="C23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D23" t="str" cm="1">
+        <f t="array" ref="D23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="E23" t="str" cm="1">
+        <f t="array" ref="E23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="F23" t="str" cm="1">
+        <f t="array" ref="F23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="G23" t="str" cm="1">
+        <f t="array" ref="G23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="H23" t="str" cm="1">
+        <f t="array" ref="H23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="I23" t="str" cm="1">
+        <f t="array" ref="I23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="J23" t="str" cm="1">
+        <f t="array" ref="J23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="K23" t="str" cm="1">
+        <f t="array" ref="K23">_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L23" t="str" cm="1">
-        <f t="array" ref="L23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
-        <v/>
+        <f t="array" ref="L23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v>Shifting cultivation</v>
       </c>
       <c r="M23" t="str" cm="1">
-        <f t="array" ref="M23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
-        <v/>
+        <f t="array" ref="M23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
+        <v>tree crop</v>
       </c>
       <c r="N23" t="str" cm="1">
-        <f t="array" ref="N23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v>other</v>
+      </c>
+      <c r="Q23" t="str" cm="1">
+        <f t="array" ref="Q23">IFERROR(_xlfn.SWITCH(VLOOKUP($A23, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="S23" t="s">
+        <v>49</v>
+      </c>
+      <c r="T23" t="s">
+        <v>39</v>
+      </c>
+      <c r="W23" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" s="8">
         <v>22</v>
       </c>
-      <c r="B24" t="e" cm="1">
-        <f t="array" ref="B24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="C24" t="e" cm="1">
-        <f t="array" ref="C24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D24" t="e" cm="1">
-        <f t="array" ref="D24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E24" t="e" cm="1">
-        <f t="array" ref="E24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F24" t="e" cm="1">
-        <f t="array" ref="F24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G24" t="e" cm="1">
-        <f t="array" ref="G24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H24" t="e" cm="1">
-        <f t="array" ref="H24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="I24" t="e" cm="1">
-        <f t="array" ref="I24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="J24" t="e" cm="1">
-        <f t="array" ref="J24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K24" t="e" cm="1">
-        <f t="array" ref="K24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$19, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
-        <v>#N/A</v>
+      <c r="B24" t="str" cm="1">
+        <f t="array" ref="B24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C24" t="str" cm="1">
+        <f t="array" ref="C24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="D24" t="str" cm="1">
+        <f t="array" ref="D24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>wetland</v>
+      </c>
+      <c r="E24" t="str" cm="1">
+        <f t="array" ref="E24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="F24" t="str" cm="1">
+        <f t="array" ref="F24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="G24" t="str" cm="1">
+        <f t="array" ref="G24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="H24" t="str" cm="1">
+        <f t="array" ref="H24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>wetland</v>
+      </c>
+      <c r="I24" t="str" cm="1">
+        <f t="array" ref="I24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="J24" t="str" cm="1">
+        <f t="array" ref="J24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="K24" t="str" cm="1">
+        <f t="array" ref="K24">_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
       </c>
       <c r="L24" t="str" cm="1">
-        <f t="array" ref="L24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$N$19, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <f t="array" ref="L24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
         <v/>
       </c>
       <c r="M24" t="str" cm="1">
-        <f t="array" ref="M24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$N$19, M$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <f t="array" ref="M24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
         <v/>
       </c>
       <c r="N24" t="str" cm="1">
-        <f t="array" ref="N24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$N$19, N$1, 0), 1, "yes"), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A25" s="8"/>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A26" s="8"/>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A27" s="8"/>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+        <f t="array" ref="N24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q24" t="str" cm="1">
+        <f t="array" ref="Q24">IFERROR(_xlfn.SWITCH(VLOOKUP($A24, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T24" t="s">
+        <v>61</v>
+      </c>
+      <c r="W24" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A25" s="8">
+        <v>23</v>
+      </c>
+      <c r="B25" t="str" cm="1">
+        <f t="array" ref="B25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, B$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="C25" t="str" cm="1">
+        <f t="array" ref="C25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, C$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="D25" t="str" cm="1">
+        <f t="array" ref="D25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, D$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>tall veg</v>
+      </c>
+      <c r="E25" t="str" cm="1">
+        <f t="array" ref="E25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, E$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>wetland</v>
+      </c>
+      <c r="F25" t="str" cm="1">
+        <f t="array" ref="F25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, F$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="G25" t="str" cm="1">
+        <f t="array" ref="G25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, G$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>wetland</v>
+      </c>
+      <c r="H25" t="str" cm="1">
+        <f t="array" ref="H25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, H$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="I25" t="str" cm="1">
+        <f t="array" ref="I25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, I$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>wetland</v>
+      </c>
+      <c r="J25" t="str" cm="1">
+        <f t="array" ref="J25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, J$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>short veg</v>
+      </c>
+      <c r="K25" t="str" cm="1">
+        <f t="array" ref="K25">_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$K$100, K$1, 0), 0, "bare", 1, "short veg", 2, "cultivated", 3, "tall veg", 4, "wetland", 5, "short veg", 6, "cultivated", 7, "tall veg", 8, "water", 9, "snow/ice", 10, "cropland", 11, "built up")</f>
+        <v>wetland</v>
+      </c>
+      <c r="L25" t="str" cm="1">
+        <f t="array" ref="L25">IFERROR(_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$P$100, L$1, 0), 1, "Permanent agriculture", 2, "Hard commodities", 3, "Shifting cultivation", 4, "Logging", 5, "Wildfire", 6, "Settlements &amp; infrastructure", 7, "Other natural disturbances"), "")</f>
+        <v/>
+      </c>
+      <c r="M25" t="str" cm="1">
+        <f t="array" ref="M25">IFERROR(_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$P$100, M$1, 0), 1, "planted forest", 2, "tree crop"), "")</f>
+        <v/>
+      </c>
+      <c r="N25" t="str" cm="1">
+        <f t="array" ref="N25">IFERROR(_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$P$100, N$1, 0), 1, "oil palm", 2, "wood fiber", 3, "other"), "")</f>
+        <v/>
+      </c>
+      <c r="Q25" t="str" cm="1">
+        <f t="array" ref="Q25">IFERROR(_xlfn.SWITCH(VLOOKUP($A25, scenarios!$A$2:$P$100, Q$1, 0), 1, "yes"), "")</f>
+        <v/>
+      </c>
+      <c r="T25" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A26" s="8">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A27" s="8">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" s="8"/>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" s="8"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" s="8"/>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" s="8"/>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
@@ -2904,19 +3375,24 @@
       <c r="A66" s="8"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:Q1 B2:K1048576">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+  <conditionalFormatting sqref="B1:K1048576">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>"wetland"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:T1 B2:K1048576">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>"short veg"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
       <formula>"tall veg"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L1:N1 B1:K1048576">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="L1:Q1 B1:K1048576">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"cropland"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"cultivated"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>